<commit_message>
data: live v2.1 market ranking
</commit_message>
<xml_diff>
--- a/reports/investment_dashboard.xlsx
+++ b/reports/investment_dashboard.xlsx
@@ -525,16 +525,16 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Micron Technology, Inc.</t>
+          <t>Taiwan Semiconductor Manufacturing Company Limited</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>57.27</v>
+        <v>55.66</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>966.780029296875</v>
+        <v>418.9500122070312</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -550,24 +550,19 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>84.2</v>
+        <v>100</v>
       </c>
       <c r="I2" t="n">
-        <v>88.2</v>
+        <v>100</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Revenue Growth; Earnings Fcf; Balance Sheet</t>
+          <t>Revenue Growth; Earnings Fcf; Balance Sheet; Valuation</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
           <t>Industry Growth; Competitive Advantage; Catalysts; Inflation Resilience</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>High market sensitivity / beta</t>
         </is>
       </c>
     </row>
@@ -577,16 +572,16 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Taiwan Semiconductor Manufacturing Company Limited</t>
+          <t>Micron Technology, Inc.</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>55.66</v>
+        <v>55.05</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -594,7 +589,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>418.9500122070312</v>
+        <v>966.780029296875</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -602,19 +597,24 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="I3" t="n">
         <v>100</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Revenue Growth; Earnings Fcf; Balance Sheet; Valuation</t>
+          <t>Revenue Growth; Earnings Fcf; Balance Sheet</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
           <t>Industry Growth; Competitive Advantage; Catalysts; Inflation Resilience</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>High market sensitivity / beta</t>
         </is>
       </c>
     </row>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MongoDB, Inc. Class A Common Stock</t>
+          <t>MongoDB, Inc.</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1426,11 +1426,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ACM Research, Inc. Class A Common Stock</t>
+          <t>ACM Research, Inc.</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>42.73</v>
+        <v>42.76</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -2115,7 +2115,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -2128,19 +2128,19 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>9.02</v>
+        <v>8.84</v>
       </c>
       <c r="F2" t="n">
-        <v>7.04</v>
+        <v>8.67</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>7.71</v>
+        <v>5.46</v>
       </c>
       <c r="I2" t="n">
-        <v>3.5</v>
+        <v>2.69</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -2149,13 +2149,13 @@
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>57.27</v>
+        <v>55.66</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -2168,19 +2168,19 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>8.84</v>
+        <v>9.02</v>
       </c>
       <c r="F3" t="n">
-        <v>8.67</v>
+        <v>4.82</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>5.46</v>
+        <v>7.71</v>
       </c>
       <c r="I3" t="n">
-        <v>2.69</v>
+        <v>3.5</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
@@ -2189,7 +2189,7 @@
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>55.66</v>
+        <v>55.05</v>
       </c>
     </row>
     <row r="4">
@@ -2851,7 +2851,7 @@
         <v>4.02</v>
       </c>
       <c r="F20" t="n">
-        <v>6.86</v>
+        <v>6.89</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
@@ -2869,7 +2869,7 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>42.73</v>
+        <v>42.76</v>
       </c>
     </row>
     <row r="21">
@@ -3343,7 +3343,7 @@
     <col width="15" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
     <col width="18" customWidth="1" min="16" max="16"/>
-    <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
     <col width="16" customWidth="1" min="18" max="18"/>
     <col width="19" customWidth="1" min="19" max="19"/>
     <col width="23" customWidth="1" min="20" max="20"/>
@@ -3514,12 +3514,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Micron Technology, Inc.</t>
+          <t>Taiwan Semiconductor Manufacturing Company Limited</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -3532,60 +3532,69 @@
           <t>Semiconductors</t>
         </is>
       </c>
+      <c r="E2" t="n">
+        <v>2172873342976</v>
+      </c>
       <c r="F2" t="n">
-        <v>966.780029296875</v>
+        <v>418.9500122070312</v>
       </c>
       <c r="G2" t="n">
-        <v>90273996800</v>
+        <v>4440492343296</v>
       </c>
       <c r="H2" t="n">
-        <v>3.457</v>
+        <v>0.36</v>
       </c>
       <c r="I2" t="n">
-        <v>44.23</v>
+        <v>13.4</v>
       </c>
       <c r="J2" t="n">
-        <v>13.685</v>
+        <v>0.774</v>
       </c>
       <c r="K2" t="n">
-        <v>7639499776</v>
+        <v>730826014720</v>
       </c>
       <c r="M2" t="n">
-        <v>26022000640</v>
+        <v>3518010228736</v>
       </c>
       <c r="N2" t="n">
-        <v>6376000000</v>
+        <v>1068558516224</v>
       </c>
       <c r="O2" t="n">
-        <v>0.7256899999999999</v>
+        <v>0.6423</v>
       </c>
       <c r="P2" t="n">
-        <v>0.80370003</v>
+        <v>0.60344005</v>
       </c>
       <c r="Q2" t="n">
-        <v>21.858015</v>
+        <v>31.264927</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0.48933163</v>
+      </c>
+      <c r="S2" t="n">
+        <v>2.97317459861974</v>
       </c>
       <c r="T2" t="n">
-        <v>0.007608338867642228</v>
+        <v>-0.005365445487747644</v>
       </c>
       <c r="U2" t="n">
-        <v>0.2875215850577266</v>
+        <v>0.03809732083456407</v>
       </c>
       <c r="V2" t="n">
-        <v>1.317802614597143</v>
+        <v>0.1684963370842598</v>
       </c>
       <c r="W2" t="n">
-        <v>7.362826824630407</v>
+        <v>0.8632972961454419</v>
       </c>
       <c r="X2" t="n">
-        <v>0.00243</v>
+        <v>0.00013</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.79989</v>
+        <v>0.155</v>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:04.075142+00:00</t>
+          <t>2026-08-22T01:53:26.879198+00:00</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
@@ -3597,12 +3606,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Taiwan Semiconductor Manufacturing Company Limited</t>
+          <t>Micron Technology, Inc.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3616,68 +3625,68 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>2172873342976</v>
+        <v>1091874717696</v>
       </c>
       <c r="F3" t="n">
-        <v>418.9500122070312</v>
+        <v>966.780029296875</v>
       </c>
       <c r="G3" t="n">
-        <v>4440492343296</v>
+        <v>90273996800</v>
       </c>
       <c r="H3" t="n">
-        <v>0.36</v>
+        <v>3.457</v>
       </c>
       <c r="I3" t="n">
-        <v>13.4</v>
+        <v>44.23</v>
       </c>
       <c r="J3" t="n">
-        <v>0.774</v>
+        <v>13.685</v>
       </c>
       <c r="K3" t="n">
-        <v>730826014720</v>
+        <v>7639499776</v>
       </c>
       <c r="M3" t="n">
-        <v>3518010228736</v>
+        <v>26022000640</v>
       </c>
       <c r="N3" t="n">
-        <v>1068558516224</v>
+        <v>6376000000</v>
       </c>
       <c r="O3" t="n">
-        <v>0.6423</v>
+        <v>0.7256899999999999</v>
       </c>
       <c r="P3" t="n">
-        <v>0.60344005</v>
+        <v>0.80370003</v>
       </c>
       <c r="Q3" t="n">
-        <v>31.264927</v>
+        <v>21.858015</v>
       </c>
       <c r="R3" t="n">
-        <v>0.48933163</v>
+        <v>12.0951185</v>
       </c>
       <c r="S3" t="n">
-        <v>2.97317459861974</v>
+        <v>142.924896879531</v>
       </c>
       <c r="T3" t="n">
-        <v>-0.005365445487747644</v>
+        <v>0.007608338867642228</v>
       </c>
       <c r="U3" t="n">
-        <v>0.03809732083456407</v>
+        <v>0.2875215850577266</v>
       </c>
       <c r="V3" t="n">
-        <v>0.1684963370842598</v>
+        <v>1.317802614597143</v>
       </c>
       <c r="W3" t="n">
-        <v>0.8632971696944793</v>
+        <v>7.362827376540883</v>
       </c>
       <c r="X3" t="n">
-        <v>0.00013</v>
+        <v>0.00243</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.155</v>
+        <v>0.79989</v>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:10.763980+00:00</t>
+          <t>2026-08-22T01:53:19.227481+00:00</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
@@ -3720,7 +3729,7 @@
         <v>1.57</v>
       </c>
       <c r="I4" t="n">
-        <v>2.5</v>
+        <v>2.49</v>
       </c>
       <c r="J4" t="n">
         <v>3.432</v>
@@ -3741,7 +3750,7 @@
         <v>0.35661998</v>
       </c>
       <c r="Q4" t="n">
-        <v>92.228004</v>
+        <v>92.5984</v>
       </c>
       <c r="R4" t="n">
         <v>32.2041</v>
@@ -3769,7 +3778,7 @@
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:05.194232+00:00</t>
+          <t>2026-08-22T01:53:20.671246+00:00</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr">
@@ -3812,7 +3821,7 @@
         <v>0.377</v>
       </c>
       <c r="I5" t="n">
-        <v>3.16</v>
+        <v>3.24</v>
       </c>
       <c r="J5" t="n">
         <v>0.357</v>
@@ -3833,7 +3842,7 @@
         <v>0.45393002</v>
       </c>
       <c r="Q5" t="n">
-        <v>59.699364</v>
+        <v>58.225307</v>
       </c>
       <c r="R5" t="n">
         <v>22.572294</v>
@@ -3861,7 +3870,7 @@
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:13.253617+00:00</t>
+          <t>2026-08-22T01:53:30.555881+00:00</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
@@ -3904,7 +3913,7 @@
         <v>0.928</v>
       </c>
       <c r="I6" t="n">
-        <v>1.17</v>
+        <v>1.21</v>
       </c>
       <c r="J6" t="n">
         <v>2.154</v>
@@ -3925,7 +3934,7 @@
         <v>0.47120997</v>
       </c>
       <c r="Q6" t="n">
-        <v>153.79488</v>
+        <v>148.71074</v>
       </c>
       <c r="R6" t="n">
         <v>70.24212</v>
@@ -3953,7 +3962,7 @@
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:01.534381+00:00</t>
+          <t>2026-08-22T01:53:15.596545+00:00</t>
         </is>
       </c>
       <c r="AD6" t="inlineStr">
@@ -3996,7 +4005,7 @@
         <v>1.039</v>
       </c>
       <c r="I7" t="n">
-        <v>7.28</v>
+        <v>7.14</v>
       </c>
       <c r="J7" t="n">
         <v>3.858</v>
@@ -4017,7 +4026,7 @@
         <v>0.33161</v>
       </c>
       <c r="Q7" t="n">
-        <v>51.612633</v>
+        <v>52.62465</v>
       </c>
       <c r="R7" t="n">
         <v>13.159287</v>
@@ -4035,7 +4044,7 @@
         <v>0.1898762435729664</v>
       </c>
       <c r="W7" t="n">
-        <v>2.446494647256825</v>
+        <v>2.446494406067634</v>
       </c>
       <c r="X7" t="n">
         <v>0.00202</v>
@@ -4045,7 +4054,7 @@
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:05.798638+00:00</t>
+          <t>2026-08-22T01:53:21.315292+00:00</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
@@ -4137,7 +4146,7 @@
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:13.873489+00:00</t>
+          <t>2026-08-22T01:53:31.303419+00:00</t>
         </is>
       </c>
       <c r="AD8" t="inlineStr">
@@ -4219,7 +4228,7 @@
         <v>0.144129303232654</v>
       </c>
       <c r="W9" t="n">
-        <v>0.2287460719461247</v>
+        <v>0.2287461792392489</v>
       </c>
       <c r="X9" t="n">
         <v>0.03991</v>
@@ -4229,7 +4238,7 @@
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:00.977695+00:00</t>
+          <t>2026-08-22T01:53:14.711548+00:00</t>
         </is>
       </c>
       <c r="AD9" t="inlineStr">
@@ -4318,7 +4327,7 @@
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:18.824707+00:00</t>
+          <t>2026-08-22T01:53:38.699827+00:00</t>
         </is>
       </c>
       <c r="AD10" t="inlineStr">
@@ -4361,7 +4370,7 @@
         <v>0.501</v>
       </c>
       <c r="I11" t="n">
-        <v>3.94</v>
+        <v>3.98</v>
       </c>
       <c r="J11" t="n">
         <v>1.595</v>
@@ -4382,7 +4391,7 @@
         <v>0.1725</v>
       </c>
       <c r="Q11" t="n">
-        <v>120.11421</v>
+        <v>118.907036</v>
       </c>
       <c r="R11" t="n">
         <v>18.704</v>
@@ -4410,7 +4419,7 @@
       </c>
       <c r="AC11" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:02.096565+00:00</t>
+          <t>2026-08-22T01:53:16.403972+00:00</t>
         </is>
       </c>
       <c r="AD11" t="inlineStr">
@@ -4492,7 +4501,7 @@
         <v>0.1400655521483041</v>
       </c>
       <c r="W12" t="n">
-        <v>0.7311824950356518</v>
+        <v>0.731182362414351</v>
       </c>
       <c r="X12" t="n">
         <v>0.01596</v>
@@ -4502,7 +4511,7 @@
       </c>
       <c r="AC12" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:08.181398+00:00</t>
+          <t>2026-08-22T01:53:23.947831+00:00</t>
         </is>
       </c>
       <c r="AD12" t="inlineStr">
@@ -4584,7 +4593,7 @@
         <v>0.3342865245955684</v>
       </c>
       <c r="W13" t="n">
-        <v>2.097116106946919</v>
+        <v>2.097116404241915</v>
       </c>
       <c r="X13" t="n">
         <v>0.00331</v>
@@ -4594,7 +4603,7 @@
       </c>
       <c r="AC13" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:03.400143+00:00</t>
+          <t>2026-08-22T01:53:18.234976+00:00</t>
         </is>
       </c>
       <c r="AD13" t="inlineStr">
@@ -4637,7 +4646,7 @@
         <v>0.356</v>
       </c>
       <c r="I14" t="n">
-        <v>0.51</v>
+        <v>0.52</v>
       </c>
       <c r="J14" t="n">
         <v>14.985</v>
@@ -4658,7 +4667,7 @@
         <v>0.00666</v>
       </c>
       <c r="Q14" t="n">
-        <v>462</v>
+        <v>453.1154</v>
       </c>
       <c r="R14" t="n">
         <v>21.328741</v>
@@ -4686,7 +4695,7 @@
       </c>
       <c r="AC14" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:16.396404+00:00</t>
+          <t>2026-08-22T01:53:34.535792+00:00</t>
         </is>
       </c>
       <c r="AD14" t="inlineStr">
@@ -4729,7 +4738,7 @@
         <v>0.479</v>
       </c>
       <c r="I15" t="n">
-        <v>6.01</v>
+        <v>6.08</v>
       </c>
       <c r="J15" t="n">
         <v>0.854</v>
@@ -4750,7 +4759,7 @@
         <v>0.48988</v>
       </c>
       <c r="Q15" t="n">
-        <v>61.306156</v>
+        <v>60.60033</v>
       </c>
       <c r="R15" t="n">
         <v>23.22839</v>
@@ -4765,7 +4774,7 @@
         <v>-0.1089169343844046</v>
       </c>
       <c r="V15" t="n">
-        <v>0.1072406716938052</v>
+        <v>0.1072405701495147</v>
       </c>
       <c r="W15" t="n">
         <v>0.2815942361128876</v>
@@ -4778,7 +4787,7 @@
       </c>
       <c r="AC15" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:02.710452+00:00</t>
+          <t>2026-08-22T01:53:17.275059+00:00</t>
         </is>
       </c>
       <c r="AD15" t="inlineStr">
@@ -4864,7 +4873,7 @@
       </c>
       <c r="AC16" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:15.802810+00:00</t>
+          <t>2026-08-22T01:53:33.581729+00:00</t>
         </is>
       </c>
       <c r="AD16" t="inlineStr">
@@ -4956,7 +4965,7 @@
       </c>
       <c r="AC17" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:08.903136+00:00</t>
+          <t>2026-08-22T01:53:24.330842+00:00</t>
         </is>
       </c>
       <c r="AD17" t="inlineStr">
@@ -4973,7 +4982,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>MongoDB, Inc. Class A Common Stock</t>
+          <t>MongoDB, Inc.</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -5042,7 +5051,7 @@
       </c>
       <c r="AC18" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:18.242316+00:00</t>
+          <t>2026-08-22T01:53:37.699969+00:00</t>
         </is>
       </c>
       <c r="AD18" t="inlineStr">
@@ -5128,7 +5137,7 @@
       </c>
       <c r="AC19" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:17.008833+00:00</t>
+          <t>2026-08-22T01:53:35.482358+00:00</t>
         </is>
       </c>
       <c r="AD19" t="inlineStr">
@@ -5145,7 +5154,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ACM Research, Inc. Class A Common Stock</t>
+          <t>ACM Research, Inc.</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -5171,7 +5180,7 @@
         <v>0.36</v>
       </c>
       <c r="I20" t="n">
-        <v>2.12</v>
+        <v>2.14</v>
       </c>
       <c r="J20" t="n">
         <v>1.806</v>
@@ -5192,7 +5201,7 @@
         <v>0.16982001</v>
       </c>
       <c r="Q20" t="n">
-        <v>37.45755</v>
+        <v>37.107475</v>
       </c>
       <c r="R20" t="n">
         <v>5.329536</v>
@@ -5217,7 +5226,7 @@
       </c>
       <c r="AC20" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:04.613522+00:00</t>
+          <t>2026-08-22T01:53:20.063957+00:00</t>
         </is>
       </c>
       <c r="AD20" t="inlineStr">
@@ -5309,7 +5318,7 @@
       </c>
       <c r="AC21" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:14.515160+00:00</t>
+          <t>2026-08-22T01:53:31.988027+00:00</t>
         </is>
       </c>
       <c r="AD21" t="inlineStr">
@@ -5401,7 +5410,7 @@
       </c>
       <c r="AC22" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:11.443345+00:00</t>
+          <t>2026-08-22T01:53:27.631839+00:00</t>
         </is>
       </c>
       <c r="AD22" t="inlineStr">
@@ -5490,7 +5499,7 @@
       </c>
       <c r="AC23" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:15.196451+00:00</t>
+          <t>2026-08-22T01:53:32.771618+00:00</t>
         </is>
       </c>
       <c r="AD23" t="inlineStr">
@@ -5533,7 +5542,7 @@
         <v>0.177</v>
       </c>
       <c r="I24" t="n">
-        <v>17.95</v>
+        <v>18.02</v>
       </c>
       <c r="J24" t="n">
         <v>0.317</v>
@@ -5554,7 +5563,7 @@
         <v>0.45111</v>
       </c>
       <c r="Q24" t="n">
-        <v>26.921446</v>
+        <v>26.81687</v>
       </c>
       <c r="R24" t="n">
         <v>10.813438</v>
@@ -5582,7 +5591,7 @@
       </c>
       <c r="AC24" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:07.555990+00:00</t>
+          <t>2026-08-22T01:53:23.183402+00:00</t>
         </is>
       </c>
       <c r="AD24" t="inlineStr">
@@ -5671,7 +5680,7 @@
       </c>
       <c r="AC25" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:06.945375+00:00</t>
+          <t>2026-08-22T01:53:22.351936+00:00</t>
         </is>
       </c>
       <c r="AD25" t="inlineStr">
@@ -5763,7 +5772,7 @@
       </c>
       <c r="AC26" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:11.995875+00:00</t>
+          <t>2026-08-22T01:53:28.756466+00:00</t>
         </is>
       </c>
       <c r="AD26" t="inlineStr">
@@ -5849,7 +5858,7 @@
       </c>
       <c r="AC27" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:06.372514+00:00</t>
+          <t>2026-08-22T01:53:21.832209+00:00</t>
         </is>
       </c>
       <c r="AD27" t="inlineStr">
@@ -5931,7 +5940,7 @@
         <v>-0.1456296261876776</v>
       </c>
       <c r="W28" t="n">
-        <v>-0.253548447765114</v>
+        <v>-0.2535483859208238</v>
       </c>
       <c r="X28" t="n">
         <v>0.00148</v>
@@ -5941,7 +5950,7 @@
       </c>
       <c r="AC28" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:09.467259+00:00</t>
+          <t>2026-08-22T01:53:25.278066+00:00</t>
         </is>
       </c>
       <c r="AD28" t="inlineStr">
@@ -6033,7 +6042,7 @@
       </c>
       <c r="AC29" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:12.703551+00:00</t>
+          <t>2026-08-22T01:53:29.696687+00:00</t>
         </is>
       </c>
       <c r="AD29" t="inlineStr">
@@ -6076,7 +6085,7 @@
         <v>0.24</v>
       </c>
       <c r="I30" t="n">
-        <v>1.6</v>
+        <v>1.58</v>
       </c>
       <c r="J30" t="n">
         <v>-0.219</v>
@@ -6097,7 +6106,7 @@
         <v>0.04063</v>
       </c>
       <c r="Q30" t="n">
-        <v>80.299995</v>
+        <v>81.31645</v>
       </c>
       <c r="R30" t="n">
         <v>9.016465999999999</v>
@@ -6125,7 +6134,7 @@
       </c>
       <c r="AC30" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:17.551468+00:00</t>
+          <t>2026-08-22T01:53:36.630899+00:00</t>
         </is>
       </c>
       <c r="AD30" t="inlineStr">
@@ -6204,7 +6213,7 @@
         <v>-0.05779410309686361</v>
       </c>
       <c r="W31" t="n">
-        <v>-0.3646448121864612</v>
+        <v>-0.3646447701327261</v>
       </c>
       <c r="X31" t="n">
         <v>0.40498</v>
@@ -6214,7 +6223,7 @@
       </c>
       <c r="AC31" t="inlineStr">
         <is>
-          <t>2026-08-22T00:21:10.135137+00:00</t>
+          <t>2026-08-22T01:53:26.086204+00:00</t>
         </is>
       </c>
       <c r="AD31" t="inlineStr">
@@ -6242,7 +6251,7 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -6299,27 +6308,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>84.2</v>
+        <v>100</v>
       </c>
       <c r="C2" t="n">
-        <v>88.2</v>
+        <v>100</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>MODERATE</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>price_to_sales, price_to_fcf</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -6333,11 +6337,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C3" t="n">
         <v>100</v>
@@ -6348,7 +6352,7 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -7285,11 +7289,11 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>57.27</v>
+        <v>55.66</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -7302,7 +7306,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>84.2</v>
+        <v>100</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
data: live v2.1 market ranking refresh
</commit_message>
<xml_diff>
--- a/reports/investment_dashboard.xlsx
+++ b/reports/investment_dashboard.xlsx
@@ -442,7 +442,7 @@
     <col width="45" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
@@ -534,15 +534,12 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>56.02</v>
+        <v>55.21</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
           <t>RESEARCH</t>
         </is>
-      </c>
-      <c r="F2" t="n">
-        <v>428.9100036621094</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -581,15 +578,12 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>54.95</v>
+        <v>53.68</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>RESEARCH</t>
         </is>
-      </c>
-      <c r="F3" t="n">
-        <v>1016.590026855469</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -633,15 +627,12 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>51.72</v>
+        <v>51.49</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>RESEARCH</t>
         </is>
-      </c>
-      <c r="F4" t="n">
-        <v>193.7799987792969</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -685,15 +676,12 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>51.57</v>
+        <v>51.29</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>RESEARCH</t>
         </is>
-      </c>
-      <c r="F5" t="n">
-        <v>230.3600006103516</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -737,16 +725,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>51.35</v>
+        <v>50.75</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
           <t>RESEARCH</t>
         </is>
       </c>
-      <c r="F6" t="n">
-        <v>524.1400146484375</v>
-      </c>
       <c r="G6" t="inlineStr">
         <is>
           <t>LOW</t>
@@ -760,7 +745,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Revenue Growth; Momentum</t>
+          <t>Revenue Growth</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -775,28 +760,25 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>TER</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Teradyne, Inc.</t>
+          <t>Palantir Technologies Inc.</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>50.61</v>
+        <v>50.19</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
           <t>RESEARCH</t>
         </is>
       </c>
-      <c r="F7" t="n">
-        <v>357.0299987792969</v>
-      </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -813,6 +795,11 @@
       <c r="K7" t="inlineStr">
         <is>
           <t>Industry Growth; Valuation; Competitive Advantage; Catalysts; Inflation Resilience</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Excessive price-to-sales valuation; Very high earnings multiple</t>
         </is>
       </c>
     </row>
@@ -822,25 +809,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Palantir Technologies Inc.</t>
+          <t>Credo Technology Group Holding Ltd</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>49.58</v>
+        <v>49.69</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
       </c>
-      <c r="F8" t="n">
-        <v>174.3300018310547</v>
-      </c>
       <c r="G8" t="inlineStr">
         <is>
           <t>MEDIUM</t>
@@ -864,7 +848,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Excessive price-to-sales valuation; Very high earnings multiple</t>
+          <t>Excessive price-to-sales valuation; High market sensitivity / beta</t>
         </is>
       </c>
     </row>
@@ -874,28 +858,25 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>TER</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Credo Technology Group Holding Ltd</t>
+          <t>Teradyne, Inc.</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>49.49</v>
+        <v>49.37</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
       </c>
-      <c r="F9" t="n">
-        <v>170.5700073242188</v>
-      </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="H9" t="n">
@@ -911,12 +892,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Industry Growth; Valuation; Competitive Advantage; Catalysts; Inflation Resilience</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>Excessive price-to-sales valuation; High market sensitivity / beta</t>
+          <t>Industry Growth; Valuation; Competitive Advantage; Momentum; Catalysts; Inflation Resilience</t>
         </is>
       </c>
     </row>
@@ -926,49 +902,41 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Advanced Micro Devices, Inc.</t>
+          <t>UiPath, Inc.</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>47.86</v>
+        <v>48.33</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
       </c>
-      <c r="F10" t="n">
-        <v>477.5700073242188</v>
-      </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>100</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="I10" t="n">
-        <v>100</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Revenue Growth; Earnings Fcf; Balance Sheet</t>
+          <t>Balance Sheet; Momentum</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Industry Growth; Valuation; Competitive Advantage; Catalysts; Inflation Resilience</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>Very high earnings multiple; High market sensitivity / beta</t>
+          <t>Industry Growth; Competitive Advantage; Catalysts; Inflation Resilience</t>
         </is>
       </c>
     </row>
@@ -978,44 +946,46 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PATH</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>UiPath, Inc.</t>
+          <t>Advanced Micro Devices, Inc.</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>46.85</v>
+        <v>46.66</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
       </c>
-      <c r="F11" t="n">
-        <v>15.1899995803833</v>
-      </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>94.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="I11" t="n">
-        <v>94.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Balance Sheet; Momentum</t>
+          <t>Revenue Growth; Earnings Fcf; Balance Sheet</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Industry Growth; Competitive Advantage; Catalysts; Inflation Resilience</t>
+          <t>Industry Growth; Valuation; Competitive Advantage; Catalysts; Inflation Resilience</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Very high earnings multiple; High market sensitivity / beta</t>
         </is>
       </c>
     </row>
@@ -1034,15 +1004,12 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>46.74</v>
+        <v>46.65</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
-      </c>
-      <c r="F12" t="n">
-        <v>338.4599914550781</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1081,15 +1048,12 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>45.41</v>
+        <v>45.34</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
-      </c>
-      <c r="F13" t="n">
-        <v>357.8949890136719</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1128,15 +1092,12 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>45.25</v>
+        <v>44.78</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
-      </c>
-      <c r="F14" t="n">
-        <v>223.5500030517578</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1180,15 +1141,12 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>45.24</v>
+        <v>44.19</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
-      </c>
-      <c r="F15" t="n">
-        <v>454.7099914550781</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1227,15 +1185,12 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>43.95</v>
+        <v>43.82</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
-      </c>
-      <c r="F16" t="n">
-        <v>212.9299926757812</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1270,24 +1225,21 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ACMR</t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ACM Research, Inc.</t>
+          <t>MongoDB, Inc.</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>43.56</v>
+        <v>43.32</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
-      </c>
-      <c r="F17" t="n">
-        <v>74.44000244140625</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1302,17 +1254,17 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Revenue Growth</t>
+          <t>Revenue Growth; Balance Sheet</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Industry Growth; Competitive Advantage; Catalysts; Inflation Resilience</t>
+          <t>Industry Growth; Valuation; Competitive Advantage; Catalysts; Inflation Resilience</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Negative free cash flow / unprofitable growth</t>
+          <t>Very high earnings multiple</t>
         </is>
       </c>
     </row>
@@ -1322,39 +1274,36 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>SNOW</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Vertiv Holdings Co</t>
+          <t>Snowflake Inc.</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>43.1</v>
+        <v>42.8</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
       </c>
-      <c r="F18" t="n">
-        <v>280.5299987792969</v>
-      </c>
       <c r="G18" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>100</v>
+        <v>88.2</v>
       </c>
       <c r="I18" t="n">
-        <v>100</v>
+        <v>88.2</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Earnings Fcf</t>
+          <t>Revenue Growth; Momentum</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1364,7 +1313,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>High market sensitivity / beta</t>
+          <t>Excessive price-to-sales valuation</t>
         </is>
       </c>
     </row>
@@ -1374,39 +1323,36 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MongoDB, Inc.</t>
+          <t>Vertiv Holdings Co</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>42.96</v>
+        <v>42.41</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
       </c>
-      <c r="F19" t="n">
-        <v>368.739990234375</v>
-      </c>
       <c r="G19" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
       <c r="H19" t="n">
-        <v>94.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="I19" t="n">
-        <v>94.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Revenue Growth; Balance Sheet</t>
+          <t>Earnings Fcf</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1416,7 +1362,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Very high earnings multiple</t>
+          <t>High market sensitivity / beta</t>
         </is>
       </c>
     </row>
@@ -1426,28 +1372,25 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Super Micro Computer, Inc.</t>
+          <t>Palo Alto Networks, Inc.</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>42.63</v>
+        <v>42.39</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
       </c>
-      <c r="F20" t="n">
-        <v>39.59000015258789</v>
-      </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="H20" t="n">
@@ -1458,17 +1401,17 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Revenue Growth; Valuation</t>
+          <t>Revenue Growth</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Industry Growth; Balance Sheet; Competitive Advantage; Catalysts; Inflation Resilience</t>
+          <t>Industry Growth; Valuation; Competitive Advantage; Catalysts; Inflation Resilience</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Negative free cash flow / unprofitable growth</t>
+          <t>Excessive price-to-sales valuation; Very high earnings multiple</t>
         </is>
       </c>
     </row>
@@ -1478,28 +1421,25 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>ACMR</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Palo Alto Networks, Inc.</t>
+          <t>ACM Research, Inc.</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>42.62</v>
+        <v>42.35</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
       </c>
-      <c r="F21" t="n">
-        <v>333.260009765625</v>
-      </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="H21" t="n">
@@ -1515,12 +1455,12 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Industry Growth; Valuation; Competitive Advantage; Catalysts; Inflation Resilience</t>
+          <t>Industry Growth; Competitive Advantage; Catalysts; Inflation Resilience</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Excessive price-to-sales valuation; Very high earnings multiple</t>
+          <t>Negative free cash flow / unprofitable growth</t>
         </is>
       </c>
     </row>
@@ -1530,49 +1470,41 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SNOW</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Snowflake Inc.</t>
+          <t>Amazon.com, Inc.</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>42.52</v>
+        <v>42.19</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
       </c>
-      <c r="F22" t="n">
-        <v>337.1799926757812</v>
-      </c>
       <c r="G22" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>88.2</v>
+        <v>100</v>
       </c>
       <c r="I22" t="n">
-        <v>88.2</v>
+        <v>100</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Revenue Growth; Momentum</t>
+          <t>Earnings Fcf</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Industry Growth; Valuation; Competitive Advantage; Catalysts; Inflation Resilience</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>Excessive price-to-sales valuation</t>
+          <t>Industry Growth; Competitive Advantage; Catalysts; Inflation Resilience</t>
         </is>
       </c>
     </row>
@@ -1582,25 +1514,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ASML Holding N.V.</t>
+          <t>Microsoft Corporation</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>42.44</v>
+        <v>41.43</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
       </c>
-      <c r="F23" t="n">
-        <v>1714.880004882812</v>
-      </c>
       <c r="G23" t="inlineStr">
         <is>
           <t>LOW</t>
@@ -1614,7 +1543,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Earnings Fcf; Balance Sheet</t>
+          <t>Earnings Fcf</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1629,25 +1558,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Amazon.com, Inc.</t>
+          <t>ASML Holding N.V.</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>42.11</v>
+        <v>41.33</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
       </c>
-      <c r="F24" t="n">
-        <v>258.510009765625</v>
-      </c>
       <c r="G24" t="inlineStr">
         <is>
           <t>LOW</t>
@@ -1661,12 +1587,12 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Earnings Fcf</t>
+          <t>Earnings Fcf; Balance Sheet</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Industry Growth; Competitive Advantage; Momentum; Catalysts; Inflation Resilience</t>
+          <t>Industry Growth; Valuation; Competitive Advantage; Catalysts; Inflation Resilience</t>
         </is>
       </c>
     </row>
@@ -1676,44 +1602,46 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Microsoft Corporation</t>
+          <t>Super Micro Computer, Inc.</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>41.11</v>
+        <v>41.23</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
       </c>
-      <c r="F25" t="n">
-        <v>499.7000122070312</v>
-      </c>
       <c r="G25" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
       <c r="H25" t="n">
-        <v>100</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="I25" t="n">
-        <v>100</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Earnings Fcf</t>
+          <t>Revenue Growth; Valuation</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Industry Growth; Valuation; Competitive Advantage; Catalysts; Inflation Resilience</t>
+          <t>Industry Growth; Balance Sheet; Competitive Advantage; Momentum; Catalysts; Inflation Resilience</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Negative free cash flow / unprofitable growth</t>
         </is>
       </c>
     </row>
@@ -1732,15 +1660,12 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>40.8</v>
+        <v>40.76</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
-      </c>
-      <c r="F26" t="n">
-        <v>278.9200134277344</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1784,15 +1709,12 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>40.52</v>
+        <v>40.09</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
-      </c>
-      <c r="F27" t="n">
-        <v>616.77001953125</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1831,15 +1753,12 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>40.22</v>
+        <v>39.98</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
-      </c>
-      <c r="F28" t="n">
-        <v>252.0899963378906</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1883,15 +1802,12 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>39.8</v>
+        <v>39.47</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
-      </c>
-      <c r="F29" t="n">
-        <v>213.1000061035156</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1935,15 +1851,12 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>35.38</v>
+        <v>35.82</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
-      </c>
-      <c r="F30" t="n">
-        <v>141.2599945068359</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1977,15 +1890,12 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>30.51</v>
+        <v>30.24</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
           <t>REJECT</t>
         </is>
-      </c>
-      <c r="F31" t="n">
-        <v>158.7799987792969</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -2137,7 +2047,7 @@
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>5.86</v>
+        <v>5.05</v>
       </c>
       <c r="I2" t="n">
         <v>2.69</v>
@@ -2149,7 +2059,7 @@
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>56.02</v>
+        <v>55.21</v>
       </c>
     </row>
     <row r="3">
@@ -2177,7 +2087,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>7.8</v>
+        <v>6.53</v>
       </c>
       <c r="I3" t="n">
         <v>3.5</v>
@@ -2189,7 +2099,7 @@
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>54.95</v>
+        <v>53.68</v>
       </c>
     </row>
     <row r="4">
@@ -2217,7 +2127,7 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>7.28</v>
+        <v>7.05</v>
       </c>
       <c r="I4" t="n">
         <v>3.63</v>
@@ -2229,7 +2139,7 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>51.72</v>
+        <v>51.49</v>
       </c>
     </row>
     <row r="5">
@@ -2257,7 +2167,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>6.25</v>
+        <v>5.97</v>
       </c>
       <c r="I5" t="n">
         <v>3.44</v>
@@ -2269,7 +2179,7 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>51.57</v>
+        <v>51.29</v>
       </c>
     </row>
     <row r="6">
@@ -2297,7 +2207,7 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>8.470000000000001</v>
+        <v>7.87</v>
       </c>
       <c r="I6" t="n">
         <v>3.54</v>
@@ -2309,13 +2219,13 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>51.35</v>
+        <v>50.75</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TER</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -2328,19 +2238,19 @@
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>8.9</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="F7" t="n">
-        <v>3.04</v>
+        <v>0.68</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>4.92</v>
+        <v>6.27</v>
       </c>
       <c r="I7" t="n">
-        <v>3.75</v>
+        <v>3.35</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -2349,38 +2259,38 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>50.61</v>
+        <v>50.19</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>15</v>
       </c>
       <c r="C8" t="n">
-        <v>15</v>
+        <v>14.2</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>9.890000000000001</v>
+        <v>9.83</v>
       </c>
       <c r="F8" t="n">
-        <v>0.68</v>
+        <v>2.5</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>5.66</v>
+        <v>4.62</v>
       </c>
       <c r="I8" t="n">
-        <v>3.35</v>
+        <v>3.54</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -2389,38 +2299,38 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>49.58</v>
+        <v>49.69</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>TER</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>15</v>
       </c>
       <c r="C9" t="n">
-        <v>14.2</v>
+        <v>15</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>9.83</v>
+        <v>8.9</v>
       </c>
       <c r="F9" t="n">
-        <v>2.5</v>
+        <v>3.04</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>4.42</v>
+        <v>3.68</v>
       </c>
       <c r="I9" t="n">
-        <v>3.54</v>
+        <v>3.75</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -2429,38 +2339,38 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>49.49</v>
+        <v>49.37</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>15</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="C10" t="n">
-        <v>12.88</v>
+        <v>9.32</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>8.77</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F10" t="n">
-        <v>1.33</v>
+        <v>7.69</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>6.43</v>
+        <v>9.51</v>
       </c>
       <c r="I10" t="n">
-        <v>3.45</v>
+        <v>3.75</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -2469,38 +2379,38 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>47.86</v>
+        <v>48.33</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PATH</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>8.359999999999999</v>
+        <v>15</v>
       </c>
       <c r="C11" t="n">
-        <v>9.32</v>
+        <v>12.88</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>9.699999999999999</v>
+        <v>8.77</v>
       </c>
       <c r="F11" t="n">
-        <v>7.69</v>
+        <v>1.33</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>8.029999999999999</v>
+        <v>5.23</v>
       </c>
       <c r="I11" t="n">
-        <v>3.75</v>
+        <v>3.45</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -2509,7 +2419,7 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>46.85</v>
+        <v>46.66</v>
       </c>
     </row>
     <row r="12">
@@ -2537,7 +2447,7 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>4.45</v>
+        <v>4.36</v>
       </c>
       <c r="I12" t="n">
         <v>3.53</v>
@@ -2549,7 +2459,7 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>46.74</v>
+        <v>46.65</v>
       </c>
     </row>
     <row r="13">
@@ -2577,7 +2487,7 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>2.92</v>
+        <v>2.85</v>
       </c>
       <c r="I13" t="n">
         <v>3.53</v>
@@ -2589,7 +2499,7 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>45.41</v>
+        <v>45.34</v>
       </c>
     </row>
     <row r="14">
@@ -2617,7 +2527,7 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>5.95</v>
+        <v>5.48</v>
       </c>
       <c r="I14" t="n">
         <v>3.53</v>
@@ -2629,7 +2539,7 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>45.25</v>
+        <v>44.78</v>
       </c>
     </row>
     <row r="15">
@@ -2657,7 +2567,7 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>5.33</v>
+        <v>4.28</v>
       </c>
       <c r="I15" t="n">
         <v>3.58</v>
@@ -2669,7 +2579,7 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>45.24</v>
+        <v>44.19</v>
       </c>
     </row>
     <row r="16">
@@ -2697,7 +2607,7 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>5.27</v>
+        <v>5.14</v>
       </c>
       <c r="I16" t="n">
         <v>3.67</v>
@@ -2709,38 +2619,38 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>43.95</v>
+        <v>43.82</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ACMR</t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>15</v>
+        <v>13.31</v>
       </c>
       <c r="C17" t="n">
-        <v>7.83</v>
+        <v>8.42</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>4.02</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="F17" t="n">
-        <v>7.14</v>
+        <v>2.27</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>5.94</v>
+        <v>5.69</v>
       </c>
       <c r="I17" t="n">
-        <v>3.63</v>
+        <v>3.74</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -2749,38 +2659,38 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>43.56</v>
+        <v>43.32</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>SNOW</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>10.91</v>
+        <v>14.44</v>
       </c>
       <c r="C18" t="n">
-        <v>13.39</v>
+        <v>7.5</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>7.41</v>
+        <v>7.58</v>
       </c>
       <c r="F18" t="n">
-        <v>2.98</v>
+        <v>0.96</v>
       </c>
       <c r="G18" t="n">
         <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>4.85</v>
+        <v>8.75</v>
       </c>
       <c r="I18" t="n">
-        <v>3.56</v>
+        <v>3.57</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -2789,38 +2699,38 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>43.1</v>
+        <v>42.8</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>13.31</v>
+        <v>10.91</v>
       </c>
       <c r="C19" t="n">
-        <v>8.42</v>
+        <v>13.39</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>9.890000000000001</v>
+        <v>7.41</v>
       </c>
       <c r="F19" t="n">
-        <v>2.27</v>
+        <v>2.98</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>5.33</v>
+        <v>4.16</v>
       </c>
       <c r="I19" t="n">
-        <v>3.74</v>
+        <v>3.56</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -2829,38 +2739,38 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>42.96</v>
+        <v>42.41</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>15</v>
+        <v>14.78</v>
       </c>
       <c r="C20" t="n">
-        <v>7.23</v>
+        <v>8.76</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>2.24</v>
+        <v>7.76</v>
       </c>
       <c r="F20" t="n">
-        <v>9.82</v>
+        <v>0.73</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>4.81</v>
+        <v>6.79</v>
       </c>
       <c r="I20" t="n">
-        <v>3.53</v>
+        <v>3.57</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -2869,38 +2779,38 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>42.63</v>
+        <v>42.39</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>ACMR</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>14.78</v>
+        <v>15</v>
       </c>
       <c r="C21" t="n">
-        <v>8.76</v>
+        <v>7.83</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>7.76</v>
+        <v>4.02</v>
       </c>
       <c r="F21" t="n">
-        <v>0.73</v>
+        <v>7.14</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>7.02</v>
+        <v>4.73</v>
       </c>
       <c r="I21" t="n">
-        <v>3.57</v>
+        <v>3.63</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -2909,38 +2819,38 @@
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>42.62</v>
+        <v>42.35</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SNOW</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>14.44</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="C22" t="n">
-        <v>7.5</v>
+        <v>12.28</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>7.58</v>
+        <v>6.64</v>
       </c>
       <c r="F22" t="n">
-        <v>0.96</v>
+        <v>6.52</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>8.470000000000001</v>
+        <v>4.06</v>
       </c>
       <c r="I22" t="n">
-        <v>3.57</v>
+        <v>3.47</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -2949,38 +2859,38 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>42.52</v>
+        <v>42.19</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>9.859999999999999</v>
+        <v>8.51</v>
       </c>
       <c r="C23" t="n">
-        <v>14.28</v>
+        <v>14.63</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>8.960000000000001</v>
+        <v>6.87</v>
       </c>
       <c r="F23" t="n">
-        <v>0.57</v>
+        <v>2.91</v>
       </c>
       <c r="G23" t="n">
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>6.02</v>
+        <v>5.06</v>
       </c>
       <c r="I23" t="n">
-        <v>2.75</v>
+        <v>3.45</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
@@ -2989,38 +2899,38 @@
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>42.44</v>
+        <v>41.43</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>9.220000000000001</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="C24" t="n">
-        <v>12.28</v>
+        <v>14.28</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
       </c>
       <c r="E24" t="n">
-        <v>6.64</v>
+        <v>8.960000000000001</v>
       </c>
       <c r="F24" t="n">
-        <v>6.52</v>
+        <v>0.57</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>3.98</v>
+        <v>4.91</v>
       </c>
       <c r="I24" t="n">
-        <v>3.47</v>
+        <v>2.75</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -3029,38 +2939,38 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>42.11</v>
+        <v>41.33</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>8.51</v>
+        <v>15</v>
       </c>
       <c r="C25" t="n">
-        <v>14.63</v>
+        <v>7.23</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>6.87</v>
+        <v>2.24</v>
       </c>
       <c r="F25" t="n">
-        <v>2.91</v>
+        <v>9.82</v>
       </c>
       <c r="G25" t="n">
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>4.74</v>
+        <v>3.41</v>
       </c>
       <c r="I25" t="n">
-        <v>3.45</v>
+        <v>3.53</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -3069,7 +2979,7 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>41.11</v>
+        <v>41.23</v>
       </c>
     </row>
     <row r="26">
@@ -3097,7 +3007,7 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>6.34</v>
+        <v>6.3</v>
       </c>
       <c r="I26" t="n">
         <v>3.64</v>
@@ -3109,7 +3019,7 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>40.8</v>
+        <v>40.76</v>
       </c>
     </row>
     <row r="27">
@@ -3137,7 +3047,7 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>2.15</v>
+        <v>1.72</v>
       </c>
       <c r="I27" t="n">
         <v>3.49</v>
@@ -3149,7 +3059,7 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>40.52</v>
+        <v>40.09</v>
       </c>
     </row>
     <row r="28">
@@ -3177,7 +3087,7 @@
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>5.31</v>
+        <v>5.07</v>
       </c>
       <c r="I28" t="n">
         <v>3.7</v>
@@ -3189,7 +3099,7 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>40.22</v>
+        <v>39.98</v>
       </c>
     </row>
     <row r="29">
@@ -3217,7 +3127,7 @@
         <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>7.66</v>
+        <v>7.33</v>
       </c>
       <c r="I29" t="n">
         <v>3.47</v>
@@ -3229,7 +3139,7 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>39.8</v>
+        <v>39.47</v>
       </c>
     </row>
     <row r="30">
@@ -3257,7 +3167,7 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>4.93</v>
+        <v>5.37</v>
       </c>
       <c r="I30" t="n">
         <v>3.57</v>
@@ -3269,7 +3179,7 @@
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>35.38</v>
+        <v>35.82</v>
       </c>
     </row>
     <row r="31">
@@ -3297,7 +3207,7 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>1.97</v>
+        <v>1.7</v>
       </c>
       <c r="I31" t="n">
         <v>3.58</v>
@@ -3309,7 +3219,7 @@
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>30.51</v>
+        <v>30.24</v>
       </c>
     </row>
   </sheetData>
@@ -3332,7 +3242,7 @@
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="37" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
@@ -3347,9 +3257,9 @@
     <col width="16" customWidth="1" min="18" max="18"/>
     <col width="19" customWidth="1" min="19" max="19"/>
     <col width="23" customWidth="1" min="20" max="20"/>
-    <col width="23" customWidth="1" min="21" max="21"/>
+    <col width="22" customWidth="1" min="21" max="21"/>
     <col width="22" customWidth="1" min="22" max="22"/>
-    <col width="23" customWidth="1" min="23" max="23"/>
+    <col width="22" customWidth="1" min="23" max="23"/>
     <col width="18" customWidth="1" min="24" max="24"/>
     <col width="24" customWidth="1" min="25" max="25"/>
     <col width="17" customWidth="1" min="26" max="26"/>
@@ -3535,9 +3445,6 @@
       <c r="E2" t="n">
         <v>2224530653184</v>
       </c>
-      <c r="F2" t="n">
-        <v>428.9100036621094</v>
-      </c>
       <c r="G2" t="n">
         <v>4440492343296</v>
       </c>
@@ -3575,16 +3482,16 @@
         <v>3.043858057018236</v>
       </c>
       <c r="T2" t="n">
-        <v>0.03601450159929809</v>
+        <v>-0.000383545453793932</v>
       </c>
       <c r="U2" t="n">
-        <v>0.03551422264981863</v>
+        <v>-0.06053546502366403</v>
       </c>
       <c r="V2" t="n">
-        <v>0.2183515192158456</v>
+        <v>0.1726845854435934</v>
       </c>
       <c r="W2" t="n">
-        <v>0.8436865432353922</v>
+        <v>0.8221267460079342</v>
       </c>
       <c r="X2" t="n">
         <v>0.00013</v>
@@ -3594,7 +3501,7 @@
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>2026-09-04T22:50:58.849744+00:00</t>
+          <t>2026-09-05T00:27:31.366239+00:00</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
@@ -3627,9 +3534,6 @@
       <c r="E3" t="n">
         <v>1148129771520</v>
       </c>
-      <c r="F3" t="n">
-        <v>1016.590026855469</v>
-      </c>
       <c r="G3" t="n">
         <v>90273996800</v>
       </c>
@@ -3667,16 +3571,16 @@
         <v>150.2886059538776</v>
       </c>
       <c r="T3" t="n">
-        <v>0.1381565222144967</v>
+        <v>0.07336416759626418</v>
       </c>
       <c r="U3" t="n">
-        <v>0.1767761689947756</v>
+        <v>-0.03784406122718531</v>
       </c>
       <c r="V3" t="n">
-        <v>1.561827279109681</v>
+        <v>1.392170087125255</v>
       </c>
       <c r="W3" t="n">
-        <v>7.197582384644518</v>
+        <v>7.083708399341603</v>
       </c>
       <c r="X3" t="n">
         <v>0.00238</v>
@@ -3686,7 +3590,7 @@
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>2026-09-04T22:50:54.108599+00:00</t>
+          <t>2026-09-05T00:27:28.275616+00:00</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
@@ -3719,9 +3623,6 @@
       <c r="E4" t="n">
         <v>244400128000</v>
       </c>
-      <c r="F4" t="n">
-        <v>193.7799987792969</v>
-      </c>
       <c r="G4" t="n">
         <v>10540800000</v>
       </c>
@@ -3759,16 +3660,16 @@
         <v>62.8033761235364</v>
       </c>
       <c r="T4" t="n">
-        <v>-0.01789062299414701</v>
+        <v>0.004881675299911681</v>
       </c>
       <c r="U4" t="n">
-        <v>0.25610937585155</v>
+        <v>0.1531835960245342</v>
       </c>
       <c r="V4" t="n">
-        <v>0.3901004825236505</v>
+        <v>0.4198620473304249</v>
       </c>
       <c r="W4" t="n">
-        <v>0.3726712565894525</v>
+        <v>0.3935070289501581</v>
       </c>
       <c r="X4" t="n">
         <v>0.17247</v>
@@ -3778,7 +3679,7 @@
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>2026-09-04T22:51:00.519446+00:00</t>
+          <t>2026-09-05T00:27:32.501999+00:00</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr">
@@ -3811,9 +3712,6 @@
       <c r="E5" t="n">
         <v>5562502742016</v>
       </c>
-      <c r="F5" t="n">
-        <v>230.3600006103516</v>
-      </c>
       <c r="G5" t="n">
         <v>302970011648</v>
       </c>
@@ -3851,16 +3749,16 @@
         <v>133.0427978908427</v>
       </c>
       <c r="T5" t="n">
-        <v>0.05081652827121852</v>
+        <v>0.07789937867628538</v>
       </c>
       <c r="U5" t="n">
-        <v>0.123159403974308</v>
+        <v>0.04477267503050575</v>
       </c>
       <c r="V5" t="n">
-        <v>0.2579959074166553</v>
+        <v>0.2496101358339837</v>
       </c>
       <c r="W5" t="n">
-        <v>0.3437423731275611</v>
+        <v>0.3407235503560528</v>
       </c>
       <c r="X5" t="n">
         <v>0.04007</v>
@@ -3870,7 +3768,7 @@
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>2026-09-04T22:50:51.754315+00:00</t>
+          <t>2026-09-05T00:27:26.674145+00:00</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
@@ -3903,9 +3801,6 @@
       <c r="E6" t="n">
         <v>338669076480</v>
       </c>
-      <c r="F6" t="n">
-        <v>524.1400146484375</v>
-      </c>
       <c r="G6" t="n">
         <v>151197007872</v>
       </c>
@@ -3943,16 +3838,16 @@
         <v>1951.983149740634</v>
       </c>
       <c r="T6" t="n">
-        <v>0.1327858241203492</v>
+        <v>0.1051212934484616</v>
       </c>
       <c r="U6" t="n">
-        <v>0.3311851479129055</v>
+        <v>0.2255498855320293</v>
       </c>
       <c r="V6" t="n">
-        <v>2.594256896884395</v>
+        <v>2.52714994047789</v>
       </c>
       <c r="W6" t="n">
-        <v>3.190567257580693</v>
+        <v>3.216822977692807</v>
       </c>
       <c r="X6" t="n">
         <v>0.07491</v>
@@ -3962,7 +3857,7 @@
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>2026-09-04T22:51:00.867681+00:00</t>
+          <t>2026-09-05T00:27:32.830240+00:00</t>
         </is>
       </c>
       <c r="AD6" t="inlineStr">
@@ -3974,12 +3869,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TER</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Teradyne, Inc.</t>
+          <t>Palantir Technologies Inc.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -3989,72 +3884,69 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Semiconductor Equipment &amp; Materials</t>
+          <t>Software - Infrastructure</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>55818338304</v>
-      </c>
-      <c r="F7" t="n">
-        <v>357.0299987792969</v>
+        <v>418925182976</v>
       </c>
       <c r="G7" t="n">
-        <v>4464031232</v>
+        <v>6155940864</v>
       </c>
       <c r="H7" t="n">
-        <v>1.039</v>
+        <v>0.928</v>
       </c>
       <c r="I7" t="n">
-        <v>7.28</v>
+        <v>1.17</v>
       </c>
       <c r="J7" t="n">
-        <v>3.858</v>
+        <v>2.154</v>
       </c>
       <c r="K7" t="n">
-        <v>437381248</v>
+        <v>2159104512</v>
       </c>
       <c r="M7" t="n">
-        <v>354828992</v>
+        <v>9409098752</v>
       </c>
       <c r="N7" t="n">
-        <v>100127000</v>
+        <v>211400000</v>
       </c>
       <c r="O7" t="n">
-        <v>0.5924199999999999</v>
+        <v>0.84796</v>
       </c>
       <c r="P7" t="n">
-        <v>0.33161</v>
+        <v>0.47120997</v>
       </c>
       <c r="Q7" t="n">
-        <v>49.04258</v>
+        <v>149</v>
       </c>
       <c r="R7" t="n">
-        <v>12.504021</v>
+        <v>68.05218000000001</v>
       </c>
       <c r="S7" t="n">
-        <v>127.6194134047557</v>
+        <v>194.0272833703383</v>
       </c>
       <c r="T7" t="n">
-        <v>-0.0831043803173972</v>
+        <v>0.1221566129954299</v>
       </c>
       <c r="U7" t="n">
-        <v>-0.002514441133463774</v>
+        <v>0.2881439852533545</v>
       </c>
       <c r="V7" t="n">
-        <v>0.1688096216930675</v>
+        <v>0.1915268351086612</v>
       </c>
       <c r="W7" t="n">
-        <v>1.998106764490561</v>
+        <v>0.1783731825146289</v>
       </c>
       <c r="X7" t="n">
-        <v>0.00202</v>
+        <v>0.03477</v>
       </c>
       <c r="Y7" t="n">
-        <v>1.00624</v>
+        <v>0.64859</v>
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>2026-09-04T22:50:55.258738+00:00</t>
+          <t>2026-09-05T00:27:27.011496+00:00</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
@@ -4066,12 +3958,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Palantir Technologies Inc.</t>
+          <t>Credo Technology Group Holding Ltd</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -4081,72 +3973,69 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Software - Infrastructure</t>
+          <t>Semiconductors</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>418925182976</v>
-      </c>
-      <c r="F8" t="n">
-        <v>174.3300018310547</v>
+        <v>32058959872</v>
       </c>
       <c r="G8" t="n">
-        <v>6155940864</v>
+        <v>1591044992</v>
       </c>
       <c r="H8" t="n">
-        <v>0.928</v>
+        <v>1.147</v>
       </c>
       <c r="I8" t="n">
-        <v>1.17</v>
+        <v>2.84</v>
       </c>
       <c r="J8" t="n">
-        <v>2.154</v>
+        <v>0.971</v>
       </c>
       <c r="K8" t="n">
-        <v>2159104512</v>
+        <v>248290880</v>
       </c>
       <c r="M8" t="n">
-        <v>9409098752</v>
+        <v>764257984</v>
       </c>
       <c r="N8" t="n">
-        <v>211400000</v>
+        <v>26205000</v>
       </c>
       <c r="O8" t="n">
-        <v>0.84796</v>
+        <v>0.67067003</v>
       </c>
       <c r="P8" t="n">
-        <v>0.47120997</v>
+        <v>0.25198</v>
       </c>
       <c r="Q8" t="n">
-        <v>149</v>
+        <v>60.059864</v>
       </c>
       <c r="R8" t="n">
-        <v>68.05218000000001</v>
+        <v>20.149626</v>
       </c>
       <c r="S8" t="n">
-        <v>194.0272833703383</v>
+        <v>129.118555913129</v>
       </c>
       <c r="T8" t="n">
-        <v>0.100359842771766</v>
+        <v>-0.3099781462995416</v>
       </c>
       <c r="U8" t="n">
-        <v>0.2862835047681325</v>
+        <v>-0.2451954107174928</v>
       </c>
       <c r="V8" t="n">
-        <v>0.1418746572469354</v>
+        <v>0.6010337107777957</v>
       </c>
       <c r="W8" t="n">
-        <v>0.1164980306936787</v>
+        <v>0.315781057833894</v>
       </c>
       <c r="X8" t="n">
-        <v>0.03477</v>
+        <v>0.09435</v>
       </c>
       <c r="Y8" t="n">
-        <v>0.64859</v>
+        <v>0.73658997</v>
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>2026-09-04T22:50:52.234211+00:00</t>
+          <t>2026-09-05T00:27:28.786496+00:00</t>
         </is>
       </c>
       <c r="AD8" t="inlineStr">
@@ -4158,12 +4047,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>TER</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Credo Technology Group Holding Ltd</t>
+          <t>Teradyne, Inc.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -4173,72 +4062,69 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Semiconductors</t>
+          <t>Semiconductor Equipment &amp; Materials</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>32058959872</v>
-      </c>
-      <c r="F9" t="n">
-        <v>170.5700073242188</v>
+        <v>55818338304</v>
       </c>
       <c r="G9" t="n">
-        <v>1591044992</v>
+        <v>4464031232</v>
       </c>
       <c r="H9" t="n">
-        <v>1.147</v>
+        <v>1.039</v>
       </c>
       <c r="I9" t="n">
-        <v>2.84</v>
+        <v>7.28</v>
       </c>
       <c r="J9" t="n">
-        <v>0.971</v>
+        <v>3.858</v>
       </c>
       <c r="K9" t="n">
-        <v>248290880</v>
+        <v>437381248</v>
       </c>
       <c r="M9" t="n">
-        <v>764257984</v>
+        <v>354828992</v>
       </c>
       <c r="N9" t="n">
-        <v>26205000</v>
+        <v>100127000</v>
       </c>
       <c r="O9" t="n">
-        <v>0.67067003</v>
+        <v>0.5924199999999999</v>
       </c>
       <c r="P9" t="n">
-        <v>0.25198</v>
+        <v>0.33161</v>
       </c>
       <c r="Q9" t="n">
-        <v>60.059864</v>
+        <v>49.04258</v>
       </c>
       <c r="R9" t="n">
-        <v>20.149626</v>
+        <v>12.504021</v>
       </c>
       <c r="S9" t="n">
-        <v>129.118555913129</v>
+        <v>127.6194134047557</v>
       </c>
       <c r="T9" t="n">
-        <v>-0.2406624065507027</v>
+        <v>-0.160992173688548</v>
       </c>
       <c r="U9" t="n">
-        <v>-0.1755521879867478</v>
+        <v>-0.1677972557431044</v>
       </c>
       <c r="V9" t="n">
-        <v>0.4865784425648676</v>
+        <v>0.1098226491139658</v>
       </c>
       <c r="W9" t="n">
-        <v>0.2729105024195428</v>
+        <v>1.837555448792994</v>
       </c>
       <c r="X9" t="n">
-        <v>0.09435</v>
+        <v>0.00202</v>
       </c>
       <c r="Y9" t="n">
-        <v>0.73658997</v>
+        <v>1.00624</v>
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>2026-09-04T22:50:54.910677+00:00</t>
+          <t>2026-09-05T00:27:29.043536+00:00</t>
         </is>
       </c>
       <c r="AD9" t="inlineStr">
@@ -4250,12 +4136,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Advanced Micro Devices, Inc.</t>
+          <t>UiPath, Inc.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -4265,72 +4151,66 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Semiconductors</t>
+          <t>Software - Infrastructure</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>779621105664</v>
-      </c>
-      <c r="F10" t="n">
-        <v>477.5700073242188</v>
+        <v>7870246400</v>
       </c>
       <c r="G10" t="n">
-        <v>41305001984</v>
+        <v>1672329984</v>
       </c>
       <c r="H10" t="n">
-        <v>0.501</v>
+        <v>0.173</v>
       </c>
       <c r="I10" t="n">
-        <v>3.92</v>
-      </c>
-      <c r="J10" t="n">
-        <v>1.595</v>
+        <v>0.67</v>
       </c>
       <c r="K10" t="n">
-        <v>8841499648</v>
+        <v>511553632</v>
       </c>
       <c r="M10" t="n">
-        <v>13111000064</v>
+        <v>1307244032</v>
       </c>
       <c r="N10" t="n">
-        <v>4276000000</v>
+        <v>83003000</v>
       </c>
       <c r="O10" t="n">
-        <v>0.55724</v>
+        <v>0.8305</v>
       </c>
       <c r="P10" t="n">
-        <v>0.1725</v>
+        <v>0.07274</v>
       </c>
       <c r="Q10" t="n">
-        <v>121.82908</v>
+        <v>22.67164</v>
       </c>
       <c r="R10" t="n">
-        <v>18.874739</v>
+        <v>4.7061563</v>
       </c>
       <c r="S10" t="n">
-        <v>88.17747403749034</v>
+        <v>15.38498782469792</v>
       </c>
       <c r="T10" t="n">
-        <v>-0.009293601456689782</v>
+        <v>0.2921984979021195</v>
       </c>
       <c r="U10" t="n">
-        <v>0.02399331515985126</v>
+        <v>0.5612681400376338</v>
       </c>
       <c r="V10" t="n">
-        <v>1.39443476877139</v>
+        <v>0.645889775577253</v>
       </c>
       <c r="W10" t="n">
-        <v>1.951789524334888</v>
+        <v>0.6746322722158122</v>
       </c>
       <c r="X10" t="n">
-        <v>0.00424</v>
+        <v>0.09236999999999999</v>
       </c>
       <c r="Y10" t="n">
-        <v>0.75447</v>
+        <v>0.91133004</v>
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>2026-09-04T22:50:52.661710+00:00</t>
+          <t>2026-09-05T00:27:34.978802+00:00</t>
         </is>
       </c>
       <c r="AD10" t="inlineStr">
@@ -4342,12 +4222,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PATH</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>UiPath, Inc.</t>
+          <t>Advanced Micro Devices, Inc.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -4357,69 +4237,69 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Software - Infrastructure</t>
+          <t>Semiconductors</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>7870246400</v>
-      </c>
-      <c r="F11" t="n">
-        <v>15.1899995803833</v>
+        <v>779621105664</v>
       </c>
       <c r="G11" t="n">
-        <v>1672329984</v>
+        <v>41305001984</v>
       </c>
       <c r="H11" t="n">
-        <v>0.173</v>
+        <v>0.501</v>
       </c>
       <c r="I11" t="n">
-        <v>0.67</v>
+        <v>3.92</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1.595</v>
       </c>
       <c r="K11" t="n">
-        <v>511553632</v>
+        <v>8841499648</v>
       </c>
       <c r="M11" t="n">
-        <v>1307244032</v>
+        <v>13111000064</v>
       </c>
       <c r="N11" t="n">
-        <v>83003000</v>
+        <v>4276000000</v>
       </c>
       <c r="O11" t="n">
-        <v>0.8305</v>
+        <v>0.55724</v>
       </c>
       <c r="P11" t="n">
-        <v>0.07274</v>
+        <v>0.1725</v>
       </c>
       <c r="Q11" t="n">
-        <v>22.67164</v>
+        <v>121.82908</v>
       </c>
       <c r="R11" t="n">
-        <v>4.7061563</v>
+        <v>18.874739</v>
       </c>
       <c r="S11" t="n">
-        <v>15.38498782469792</v>
+        <v>88.17747403749034</v>
       </c>
       <c r="T11" t="n">
-        <v>0.09913168710648868</v>
+        <v>-0.1203671783922984</v>
       </c>
       <c r="U11" t="n">
-        <v>0.3514234777312801</v>
+        <v>-0.1281345699173914</v>
       </c>
       <c r="V11" t="n">
-        <v>0.3151514571028631</v>
+        <v>1.257435478438948</v>
       </c>
       <c r="W11" t="n">
-        <v>0.3999999121037527</v>
+        <v>1.813544624215744</v>
       </c>
       <c r="X11" t="n">
-        <v>0.09236999999999999</v>
+        <v>0.00424</v>
       </c>
       <c r="Y11" t="n">
-        <v>0.91133004</v>
+        <v>0.75447</v>
       </c>
       <c r="AC11" t="inlineStr">
         <is>
-          <t>2026-09-04T22:51:04.085597+00:00</t>
+          <t>2026-09-05T00:27:27.308147+00:00</t>
         </is>
       </c>
       <c r="AD11" t="inlineStr">
@@ -4452,9 +4332,6 @@
       <c r="E12" t="n">
         <v>4139343675392</v>
       </c>
-      <c r="F12" t="n">
-        <v>338.4599914550781</v>
-      </c>
       <c r="G12" t="n">
         <v>445865984000</v>
       </c>
@@ -4492,16 +4369,16 @@
         <v>182.6315243796928</v>
       </c>
       <c r="T12" t="n">
-        <v>-0.06613691390090326</v>
+        <v>-0.09312851444079862</v>
       </c>
       <c r="U12" t="n">
-        <v>-0.08104587521756546</v>
+        <v>-0.07927519735176403</v>
       </c>
       <c r="V12" t="n">
-        <v>0.1263644045246901</v>
+        <v>0.1312828803719981</v>
       </c>
       <c r="W12" t="n">
-        <v>0.4611517712780797</v>
+        <v>0.4890185333458321</v>
       </c>
       <c r="X12" t="n">
         <v>0.01596</v>
@@ -4511,7 +4388,7 @@
       </c>
       <c r="AC12" t="inlineStr">
         <is>
-          <t>2026-09-04T22:50:57.091067+00:00</t>
+          <t>2026-09-05T00:27:30.199474+00:00</t>
         </is>
       </c>
       <c r="AD12" t="inlineStr">
@@ -4544,9 +4421,6 @@
       <c r="E13" t="n">
         <v>1702714146816</v>
       </c>
-      <c r="F13" t="n">
-        <v>357.8949890136719</v>
-      </c>
       <c r="G13" t="n">
         <v>89103998976</v>
       </c>
@@ -4584,16 +4458,16 @@
         <v>55.83195737287067</v>
       </c>
       <c r="T13" t="n">
-        <v>-0.1443650424162088</v>
+        <v>-0.1458771749229525</v>
       </c>
       <c r="U13" t="n">
-        <v>-0.07069344674819256</v>
+        <v>-0.1460569718599254</v>
       </c>
       <c r="V13" t="n">
-        <v>0.0794644900225383</v>
+        <v>0.1289505100786794</v>
       </c>
       <c r="W13" t="n">
-        <v>0.1777763427651158</v>
+        <v>0.1897778733840267</v>
       </c>
       <c r="X13" t="n">
         <v>0.01948</v>
@@ -4603,7 +4477,7 @@
       </c>
       <c r="AC13" t="inlineStr">
         <is>
-          <t>2026-09-04T22:50:53.212488+00:00</t>
+          <t>2026-09-05T00:27:27.581201+00:00</t>
         </is>
       </c>
       <c r="AD13" t="inlineStr">
@@ -4636,9 +4510,6 @@
       <c r="E14" t="n">
         <v>200905424896</v>
       </c>
-      <c r="F14" t="n">
-        <v>223.5500030517578</v>
-      </c>
       <c r="G14" t="n">
         <v>9450300416</v>
       </c>
@@ -4676,16 +4547,16 @@
         <v>83.43075582752039</v>
       </c>
       <c r="T14" t="n">
-        <v>0.05937825099803629</v>
+        <v>-0.04464977661534519</v>
       </c>
       <c r="U14" t="n">
-        <v>-0.1513070056084538</v>
+        <v>-0.3398808013064741</v>
       </c>
       <c r="V14" t="n">
-        <v>1.956092444795619</v>
+        <v>1.676220852878165</v>
       </c>
       <c r="W14" t="n">
-        <v>2.494950084105129</v>
+        <v>2.35860892620654</v>
       </c>
       <c r="X14" t="n">
         <v>0.00494</v>
@@ -4695,7 +4566,7 @@
       </c>
       <c r="AC14" t="inlineStr">
         <is>
-          <t>2026-09-04T22:51:00.140734+00:00</t>
+          <t>2026-09-05T00:27:32.239527+00:00</t>
         </is>
       </c>
       <c r="AD14" t="inlineStr">
@@ -4728,9 +4599,6 @@
       <c r="E15" t="n">
         <v>360856682496</v>
       </c>
-      <c r="F15" t="n">
-        <v>454.7099914550781</v>
-      </c>
       <c r="G15" t="n">
         <v>30837000192</v>
       </c>
@@ -4768,16 +4636,16 @@
         <v>117.3374532513612</v>
       </c>
       <c r="T15" t="n">
-        <v>-0.147955519201504</v>
+        <v>-0.2016828604055149</v>
       </c>
       <c r="U15" t="n">
-        <v>0.004825949921960504</v>
+        <v>-0.1302050901264671</v>
       </c>
       <c r="V15" t="n">
-        <v>0.3152168943060754</v>
+        <v>0.2212617148845017</v>
       </c>
       <c r="W15" t="n">
-        <v>1.889440147272866</v>
+        <v>1.805254567261285</v>
       </c>
       <c r="X15" t="n">
         <v>0.0033000002</v>
@@ -4787,7 +4655,7 @@
       </c>
       <c r="AC15" t="inlineStr">
         <is>
-          <t>2026-09-04T22:50:53.694400+00:00</t>
+          <t>2026-09-05T00:27:27.971324+00:00</t>
         </is>
       </c>
       <c r="AD15" t="inlineStr">
@@ -4820,9 +4688,6 @@
       <c r="E16" t="n">
         <v>76457836544</v>
       </c>
-      <c r="F16" t="n">
-        <v>212.9299926757812</v>
-      </c>
       <c r="G16" t="n">
         <v>3966725120</v>
       </c>
@@ -4860,16 +4725,16 @@
         <v>72.7191728331531</v>
       </c>
       <c r="T16" t="n">
-        <v>-0.2480489367560754</v>
+        <v>-0.2546937391781213</v>
       </c>
       <c r="U16" t="n">
-        <v>-0.09047032539981892</v>
+        <v>-0.1183908492367787</v>
       </c>
       <c r="V16" t="n">
-        <v>0.7401928049497537</v>
+        <v>0.814924289559793</v>
       </c>
       <c r="W16" t="n">
-        <v>0.6157990184261053</v>
+        <v>0.6196077271608964</v>
       </c>
       <c r="X16" t="n">
         <v>0.00619</v>
@@ -4879,7 +4744,7 @@
       </c>
       <c r="AC16" t="inlineStr">
         <is>
-          <t>2026-09-04T22:51:02.392257+00:00</t>
+          <t>2026-09-05T00:27:33.956089+00:00</t>
         </is>
       </c>
       <c r="AD16" t="inlineStr">
@@ -4891,12 +4756,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ACMR</t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ACM Research, Inc.</t>
+          <t>MongoDB, Inc.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -4906,69 +4771,66 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Semiconductor Equipment &amp; Materials</t>
+          <t>Software - Infrastructure</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>5184686592</v>
-      </c>
-      <c r="F17" t="n">
-        <v>74.44000244140625</v>
+        <v>29658468352</v>
       </c>
       <c r="G17" t="n">
-        <v>1037772032</v>
+        <v>2782769920</v>
       </c>
       <c r="H17" t="n">
-        <v>0.36</v>
+        <v>0.305</v>
       </c>
       <c r="I17" t="n">
-        <v>2.12</v>
-      </c>
-      <c r="J17" t="n">
-        <v>1.806</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="K17" t="n">
-        <v>-186610256</v>
+        <v>561356224</v>
       </c>
       <c r="M17" t="n">
-        <v>1439374976</v>
+        <v>2411254016</v>
       </c>
       <c r="N17" t="n">
-        <v>349319008</v>
+        <v>55013000</v>
       </c>
       <c r="O17" t="n">
-        <v>0.43835</v>
+        <v>0.72688</v>
       </c>
       <c r="P17" t="n">
-        <v>0.16982001</v>
+        <v>0.0368</v>
       </c>
       <c r="Q17" t="n">
-        <v>35.11321</v>
+        <v>534.40576</v>
       </c>
       <c r="R17" t="n">
-        <v>4.9959784</v>
+        <v>10.657894</v>
+      </c>
+      <c r="S17" t="n">
+        <v>52.83359671451688</v>
       </c>
       <c r="T17" t="n">
-        <v>-0.06833540651065206</v>
+        <v>0.01160405105503015</v>
       </c>
       <c r="U17" t="n">
-        <v>-0.02424955370192639</v>
+        <v>0.01123157350074311</v>
       </c>
       <c r="V17" t="n">
-        <v>0.5408818117434713</v>
+        <v>0.5501391908479503</v>
       </c>
       <c r="W17" t="n">
-        <v>1.759080937895229</v>
+        <v>0.2287458648916376</v>
       </c>
       <c r="X17" t="n">
-        <v>0.12675999</v>
+        <v>0.02637</v>
       </c>
       <c r="Y17" t="n">
-        <v>0.77925</v>
+        <v>0.96739995</v>
       </c>
       <c r="AC17" t="inlineStr">
         <is>
-          <t>2026-09-04T22:50:54.554252+00:00</t>
+          <t>2026-09-05T00:27:34.735926+00:00</t>
         </is>
       </c>
       <c r="AD17" t="inlineStr">
@@ -4980,87 +4842,78 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>SNOW</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Vertiv Holdings Co</t>
+          <t>Snowflake Inc.</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Electrical Equipment &amp; Parts</t>
+          <t>Software - Application</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>108000731136</v>
-      </c>
-      <c r="F18" t="n">
-        <v>280.5299987792969</v>
+        <v>116866588672</v>
       </c>
       <c r="G18" t="n">
-        <v>11479600128</v>
+        <v>5032822784</v>
       </c>
       <c r="H18" t="n">
-        <v>0.241</v>
+        <v>0.335</v>
       </c>
       <c r="I18" t="n">
-        <v>4.41</v>
-      </c>
-      <c r="J18" t="n">
-        <v>0.53</v>
+        <v>-3.17</v>
       </c>
       <c r="K18" t="n">
-        <v>2696537600</v>
+        <v>1739497728</v>
       </c>
       <c r="M18" t="n">
-        <v>3110599936</v>
+        <v>2954998016</v>
       </c>
       <c r="N18" t="n">
-        <v>3338200064</v>
+        <v>2772094976</v>
       </c>
       <c r="O18" t="n">
-        <v>0.38039002</v>
+        <v>0.67144996</v>
       </c>
       <c r="P18" t="n">
-        <v>0.20362</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>63.612247</v>
+        <v>-0.22173999</v>
       </c>
       <c r="R18" t="n">
-        <v>9.408056999999999</v>
+        <v>23.220882</v>
       </c>
       <c r="S18" t="n">
-        <v>40.05163181703826</v>
+        <v>67.18409963453543</v>
       </c>
       <c r="T18" t="n">
-        <v>0.009318544704397524</v>
+        <v>0.1253275675850649</v>
       </c>
       <c r="U18" t="n">
-        <v>-0.06629281434838818</v>
+        <v>0.4598657216523836</v>
       </c>
       <c r="V18" t="n">
-        <v>0.1237443626550756</v>
+        <v>1.118566580639112</v>
       </c>
       <c r="W18" t="n">
-        <v>1.234200542459901</v>
+        <v>0.5543975859003014</v>
       </c>
       <c r="X18" t="n">
-        <v>0.00269</v>
+        <v>0.02962</v>
       </c>
       <c r="Y18" t="n">
-        <v>0.84453005</v>
+        <v>0.82354</v>
       </c>
       <c r="AC18" t="inlineStr">
         <is>
-          <t>2026-09-04T22:51:01.302180+00:00</t>
+          <t>2026-09-05T00:27:33.649651+00:00</t>
         </is>
       </c>
       <c r="AD18" t="inlineStr">
@@ -5072,84 +4925,84 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>MongoDB, Inc.</t>
+          <t>Vertiv Holdings Co</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Software - Infrastructure</t>
+          <t>Electrical Equipment &amp; Parts</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>29658468352</v>
-      </c>
-      <c r="F19" t="n">
-        <v>368.739990234375</v>
+        <v>108000731136</v>
       </c>
       <c r="G19" t="n">
-        <v>2782769920</v>
+        <v>11479600128</v>
       </c>
       <c r="H19" t="n">
-        <v>0.305</v>
+        <v>0.241</v>
       </c>
       <c r="I19" t="n">
-        <v>0.6899999999999999</v>
+        <v>4.41</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.53</v>
       </c>
       <c r="K19" t="n">
-        <v>561356224</v>
+        <v>2696537600</v>
       </c>
       <c r="M19" t="n">
-        <v>2411254016</v>
+        <v>3110599936</v>
       </c>
       <c r="N19" t="n">
-        <v>55013000</v>
+        <v>3338200064</v>
       </c>
       <c r="O19" t="n">
-        <v>0.72688</v>
+        <v>0.38039002</v>
       </c>
       <c r="P19" t="n">
-        <v>0.0368</v>
+        <v>0.20362</v>
       </c>
       <c r="Q19" t="n">
-        <v>534.40576</v>
+        <v>63.612247</v>
       </c>
       <c r="R19" t="n">
-        <v>10.657894</v>
+        <v>9.408056999999999</v>
       </c>
       <c r="S19" t="n">
-        <v>52.83359671451688</v>
+        <v>40.05163181703826</v>
       </c>
       <c r="T19" t="n">
-        <v>-0.02024656024489313</v>
+        <v>-0.004075153311462021</v>
       </c>
       <c r="U19" t="n">
-        <v>0.05132006757476337</v>
+        <v>-0.1699002535148172</v>
       </c>
       <c r="V19" t="n">
-        <v>0.3971128726068855</v>
+        <v>0.07031961217804295</v>
       </c>
       <c r="W19" t="n">
-        <v>0.1449775010437855</v>
+        <v>1.142894657238017</v>
       </c>
       <c r="X19" t="n">
-        <v>0.02637</v>
+        <v>0.00269</v>
       </c>
       <c r="Y19" t="n">
-        <v>0.96739995</v>
+        <v>0.84453005</v>
       </c>
       <c r="AC19" t="inlineStr">
         <is>
-          <t>2026-09-04T22:51:03.629921+00:00</t>
+          <t>2026-09-05T00:27:33.085590+00:00</t>
         </is>
       </c>
       <c r="AD19" t="inlineStr">
@@ -5161,12 +5014,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Super Micro Computer, Inc.</t>
+          <t>Palo Alto Networks, Inc.</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -5176,69 +5029,66 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Computer Hardware</t>
+          <t>Software - Infrastructure</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>26009260032</v>
-      </c>
-      <c r="F20" t="n">
-        <v>39.59000015258789</v>
+        <v>271606906880</v>
       </c>
       <c r="G20" t="n">
-        <v>39063072768</v>
+        <v>11480000512</v>
       </c>
       <c r="H20" t="n">
-        <v>0.9320000000000001</v>
+        <v>0.344</v>
       </c>
       <c r="I20" t="n">
-        <v>3.26</v>
-      </c>
-      <c r="J20" t="n">
-        <v>4.347</v>
+        <v>1.16</v>
       </c>
       <c r="K20" t="n">
-        <v>-8248783872</v>
+        <v>4469550080</v>
       </c>
       <c r="M20" t="n">
-        <v>7544584192</v>
+        <v>3071000064</v>
       </c>
       <c r="N20" t="n">
-        <v>9259886592</v>
+        <v>2500000000</v>
       </c>
       <c r="O20" t="n">
-        <v>0.108219996</v>
+        <v>0.70488</v>
       </c>
       <c r="P20" t="n">
-        <v>0.13382</v>
+        <v>0.050440002</v>
       </c>
       <c r="Q20" t="n">
-        <v>12.144172</v>
+        <v>287.29312</v>
       </c>
       <c r="R20" t="n">
-        <v>0.6658273</v>
+        <v>23.659138</v>
+      </c>
+      <c r="S20" t="n">
+        <v>60.76828808684027</v>
       </c>
       <c r="T20" t="n">
-        <v>0.3057388044547411</v>
+        <v>-0.09390182409882386</v>
       </c>
       <c r="U20" t="n">
-        <v>-0.04923149056457887</v>
+        <v>0.1886839836755818</v>
       </c>
       <c r="V20" t="n">
-        <v>0.2279776082961615</v>
+        <v>1.093466243393087</v>
       </c>
       <c r="W20" t="n">
-        <v>-0.02727274175784056</v>
+        <v>0.7330966666162104</v>
       </c>
       <c r="X20" t="n">
-        <v>0.12726</v>
+        <v>0.0076</v>
       </c>
       <c r="Y20" t="n">
-        <v>0.69521004</v>
+        <v>0.84849</v>
       </c>
       <c r="AC20" t="inlineStr">
         <is>
-          <t>2026-09-04T22:51:01.677205+00:00</t>
+          <t>2026-09-05T00:27:29.625919+00:00</t>
         </is>
       </c>
       <c r="AD20" t="inlineStr">
@@ -5250,12 +5100,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>ACMR</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Palo Alto Networks, Inc.</t>
+          <t>ACM Research, Inc.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -5265,69 +5115,66 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Software - Infrastructure</t>
+          <t>Semiconductor Equipment &amp; Materials</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>271606906880</v>
-      </c>
-      <c r="F21" t="n">
-        <v>333.260009765625</v>
+        <v>5184686592</v>
       </c>
       <c r="G21" t="n">
-        <v>11480000512</v>
+        <v>1037772032</v>
       </c>
       <c r="H21" t="n">
-        <v>0.344</v>
+        <v>0.36</v>
       </c>
       <c r="I21" t="n">
-        <v>1.16</v>
+        <v>2.12</v>
+      </c>
+      <c r="J21" t="n">
+        <v>1.806</v>
       </c>
       <c r="K21" t="n">
-        <v>4469550080</v>
+        <v>-186610256</v>
       </c>
       <c r="M21" t="n">
-        <v>3071000064</v>
+        <v>1439374976</v>
       </c>
       <c r="N21" t="n">
-        <v>2500000000</v>
+        <v>349319008</v>
       </c>
       <c r="O21" t="n">
-        <v>0.70488</v>
+        <v>0.43835</v>
       </c>
       <c r="P21" t="n">
-        <v>0.050440002</v>
+        <v>0.16982001</v>
       </c>
       <c r="Q21" t="n">
-        <v>287.29312</v>
+        <v>35.11321</v>
       </c>
       <c r="R21" t="n">
-        <v>23.659138</v>
-      </c>
-      <c r="S21" t="n">
-        <v>60.76828808684027</v>
+        <v>4.9959784</v>
       </c>
       <c r="T21" t="n">
-        <v>-0.08106764903657915</v>
+        <v>-0.1586474806493464</v>
       </c>
       <c r="U21" t="n">
-        <v>0.2249954961190344</v>
+        <v>-0.2304196357208406</v>
       </c>
       <c r="V21" t="n">
-        <v>1.042534949041668</v>
+        <v>0.339637178266502</v>
       </c>
       <c r="W21" t="n">
-        <v>0.7325708302097835</v>
+        <v>1.587402100870236</v>
       </c>
       <c r="X21" t="n">
-        <v>0.0076</v>
+        <v>0.12675999</v>
       </c>
       <c r="Y21" t="n">
-        <v>0.84849</v>
+        <v>0.77925</v>
       </c>
       <c r="AC21" t="inlineStr">
         <is>
-          <t>2026-09-04T22:50:56.137999+00:00</t>
+          <t>2026-09-05T00:27:28.546988+00:00</t>
         </is>
       </c>
       <c r="AD21" t="inlineStr">
@@ -5339,81 +5186,84 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SNOW</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Snowflake Inc.</t>
+          <t>Amazon.com, Inc.</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Software - Application</t>
+          <t>Internet Retail</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>116866588672</v>
-      </c>
-      <c r="F22" t="n">
-        <v>337.1799926757812</v>
+        <v>2788369891328</v>
       </c>
       <c r="G22" t="n">
-        <v>5032822784</v>
+        <v>775680032768</v>
       </c>
       <c r="H22" t="n">
-        <v>0.335</v>
+        <v>0.196</v>
       </c>
       <c r="I22" t="n">
-        <v>-3.17</v>
+        <v>12.43</v>
+      </c>
+      <c r="J22" t="n">
+        <v>2.423</v>
       </c>
       <c r="K22" t="n">
-        <v>1739497728</v>
+        <v>3219124992</v>
       </c>
       <c r="M22" t="n">
-        <v>2954998016</v>
+        <v>122988003328</v>
       </c>
       <c r="N22" t="n">
-        <v>2772094976</v>
+        <v>251635007488</v>
       </c>
       <c r="O22" t="n">
-        <v>0.67144996</v>
+        <v>0.5077</v>
       </c>
       <c r="P22" t="n">
-        <v>-0.22173999</v>
+        <v>0.13689</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>20.797264</v>
       </c>
       <c r="R22" t="n">
-        <v>23.220882</v>
+        <v>3.5947423</v>
       </c>
       <c r="S22" t="n">
-        <v>67.18409963453543</v>
+        <v>866.1887619329818</v>
       </c>
       <c r="T22" t="n">
-        <v>0.06419642902722189</v>
+        <v>-0.06675805145570113</v>
       </c>
       <c r="U22" t="n">
-        <v>0.4151766996121005</v>
+        <v>0.02013476002022796</v>
       </c>
       <c r="V22" t="n">
-        <v>0.9001408761597691</v>
+        <v>0.1940779685951302</v>
       </c>
       <c r="W22" t="n">
-        <v>0.5195133030651393</v>
+        <v>0.1456258577962457</v>
       </c>
       <c r="X22" t="n">
-        <v>0.02962</v>
+        <v>0.08866</v>
       </c>
       <c r="Y22" t="n">
-        <v>0.82354</v>
+        <v>0.68738997</v>
       </c>
       <c r="AC22" t="inlineStr">
         <is>
-          <t>2026-09-04T22:51:02.016494+00:00</t>
+          <t>2026-09-05T00:27:30.430711+00:00</t>
         </is>
       </c>
       <c r="AD22" t="inlineStr">
@@ -5425,12 +5275,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ASML Holding N.V.</t>
+          <t>Microsoft Corporation</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -5440,72 +5290,69 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Semiconductor Equipment &amp; Materials</t>
+          <t>Software - Infrastructure</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>658685427712</v>
-      </c>
-      <c r="F23" t="n">
-        <v>1714.880004882812</v>
+        <v>3710545297408</v>
       </c>
       <c r="G23" t="n">
-        <v>35327500288</v>
+        <v>331839012864</v>
       </c>
       <c r="H23" t="n">
-        <v>0.213</v>
+        <v>0.177</v>
       </c>
       <c r="I23" t="n">
-        <v>29.47</v>
+        <v>17.96</v>
       </c>
       <c r="J23" t="n">
-        <v>0.285</v>
+        <v>0.317</v>
       </c>
       <c r="K23" t="n">
-        <v>8437675008</v>
+        <v>16545500160</v>
       </c>
       <c r="M23" t="n">
-        <v>7581499904</v>
+        <v>76842999808</v>
       </c>
       <c r="N23" t="n">
-        <v>1984400000</v>
+        <v>128812998656</v>
       </c>
       <c r="O23" t="n">
-        <v>0.5273300400000001</v>
+        <v>0.67944</v>
       </c>
       <c r="P23" t="n">
-        <v>0.37057</v>
+        <v>0.45111</v>
       </c>
       <c r="Q23" t="n">
-        <v>58.190704</v>
+        <v>27.822943</v>
       </c>
       <c r="R23" t="n">
-        <v>18.645119</v>
+        <v>11.181764</v>
       </c>
       <c r="S23" t="n">
-        <v>78.06480186632947</v>
+        <v>224.2631084902785</v>
       </c>
       <c r="T23" t="n">
-        <v>0.02184459416504736</v>
+        <v>0.03707370169206503</v>
       </c>
       <c r="U23" t="n">
-        <v>0.04590119703571305</v>
+        <v>0.1939733944038662</v>
       </c>
       <c r="V23" t="n">
-        <v>0.2575991696869864</v>
+        <v>0.2640356128143941</v>
       </c>
       <c r="W23" t="n">
-        <v>1.29108903770179</v>
+        <v>0.01774439203186762</v>
       </c>
       <c r="X23" t="n">
-        <v>0.00016000001</v>
+        <v>0.00091</v>
       </c>
       <c r="Y23" t="n">
-        <v>0.20382</v>
+        <v>0.75858</v>
       </c>
       <c r="AC23" t="inlineStr">
         <is>
-          <t>2026-09-04T22:50:59.293087+00:00</t>
+          <t>2026-09-05T00:27:29.897959+00:00</t>
         </is>
       </c>
       <c r="AD23" t="inlineStr">
@@ -5517,87 +5364,84 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Amazon.com, Inc.</t>
+          <t>ASML Holding N.V.</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Internet Retail</t>
+          <t>Semiconductor Equipment &amp; Materials</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>2788369891328</v>
-      </c>
-      <c r="F24" t="n">
-        <v>258.510009765625</v>
+        <v>658685427712</v>
       </c>
       <c r="G24" t="n">
-        <v>775680032768</v>
+        <v>35327500288</v>
       </c>
       <c r="H24" t="n">
-        <v>0.196</v>
+        <v>0.213</v>
       </c>
       <c r="I24" t="n">
-        <v>12.43</v>
+        <v>29.47</v>
       </c>
       <c r="J24" t="n">
-        <v>2.423</v>
+        <v>0.285</v>
       </c>
       <c r="K24" t="n">
-        <v>3219124992</v>
+        <v>8437675008</v>
       </c>
       <c r="M24" t="n">
-        <v>122988003328</v>
+        <v>7581499904</v>
       </c>
       <c r="N24" t="n">
-        <v>251635007488</v>
+        <v>1984400000</v>
       </c>
       <c r="O24" t="n">
-        <v>0.5077</v>
+        <v>0.5273300400000001</v>
       </c>
       <c r="P24" t="n">
-        <v>0.13689</v>
+        <v>0.37057</v>
       </c>
       <c r="Q24" t="n">
-        <v>20.797264</v>
+        <v>58.190704</v>
       </c>
       <c r="R24" t="n">
-        <v>3.5947423</v>
+        <v>18.645119</v>
       </c>
       <c r="S24" t="n">
-        <v>866.1887619329818</v>
+        <v>78.06480186632947</v>
       </c>
       <c r="T24" t="n">
-        <v>-0.05186130367649244</v>
+        <v>-0.03837867659721117</v>
       </c>
       <c r="U24" t="n">
-        <v>0.05072556618399782</v>
+        <v>-0.06210688969814715</v>
       </c>
       <c r="V24" t="n">
-        <v>0.1807344792316272</v>
+        <v>0.1804735343858654</v>
       </c>
       <c r="W24" t="n">
-        <v>0.0968687109611821</v>
+        <v>1.24889767544827</v>
       </c>
       <c r="X24" t="n">
-        <v>0.08866</v>
+        <v>0.00016000001</v>
       </c>
       <c r="Y24" t="n">
-        <v>0.68738997</v>
+        <v>0.20382</v>
       </c>
       <c r="AC24" t="inlineStr">
         <is>
-          <t>2026-09-04T22:50:57.401209+00:00</t>
+          <t>2026-09-05T00:27:31.635879+00:00</t>
         </is>
       </c>
       <c r="AD24" t="inlineStr">
@@ -5609,12 +5453,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Microsoft Corporation</t>
+          <t>Super Micro Computer, Inc.</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -5624,72 +5468,66 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Software - Infrastructure</t>
+          <t>Computer Hardware</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>3710545297408</v>
-      </c>
-      <c r="F25" t="n">
-        <v>499.7000122070312</v>
+        <v>26009260032</v>
       </c>
       <c r="G25" t="n">
-        <v>331839012864</v>
+        <v>39063072768</v>
       </c>
       <c r="H25" t="n">
-        <v>0.177</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="I25" t="n">
-        <v>17.96</v>
+        <v>3.26</v>
       </c>
       <c r="J25" t="n">
-        <v>0.317</v>
+        <v>4.347</v>
       </c>
       <c r="K25" t="n">
-        <v>16545500160</v>
+        <v>-8248783872</v>
       </c>
       <c r="M25" t="n">
-        <v>76842999808</v>
+        <v>7544584192</v>
       </c>
       <c r="N25" t="n">
-        <v>128812998656</v>
+        <v>9259886592</v>
       </c>
       <c r="O25" t="n">
-        <v>0.67944</v>
+        <v>0.108219996</v>
       </c>
       <c r="P25" t="n">
-        <v>0.45111</v>
+        <v>0.13382</v>
       </c>
       <c r="Q25" t="n">
-        <v>27.822943</v>
+        <v>12.144172</v>
       </c>
       <c r="R25" t="n">
-        <v>11.181764</v>
-      </c>
-      <c r="S25" t="n">
-        <v>224.2631084902785</v>
+        <v>0.6658273</v>
       </c>
       <c r="T25" t="n">
-        <v>0.02703957504812737</v>
+        <v>0.1950141462189448</v>
       </c>
       <c r="U25" t="n">
-        <v>0.2015280836479112</v>
+        <v>-0.1925373624777279</v>
       </c>
       <c r="V25" t="n">
-        <v>0.2216934208082806</v>
+        <v>0.1598774015942512</v>
       </c>
       <c r="W25" t="n">
-        <v>-0.008186765687858366</v>
+        <v>-0.05561096326912529</v>
       </c>
       <c r="X25" t="n">
-        <v>0.00091</v>
+        <v>0.12726</v>
       </c>
       <c r="Y25" t="n">
-        <v>0.75858</v>
+        <v>0.69521004</v>
       </c>
       <c r="AC25" t="inlineStr">
         <is>
-          <t>2026-09-04T22:50:56.654412+00:00</t>
+          <t>2026-09-05T00:27:33.362654+00:00</t>
         </is>
       </c>
       <c r="AD25" t="inlineStr">
@@ -5722,9 +5560,6 @@
       <c r="E26" t="n">
         <v>99317760000</v>
       </c>
-      <c r="F26" t="n">
-        <v>278.9200134277344</v>
-      </c>
       <c r="G26" t="n">
         <v>2512349952</v>
       </c>
@@ -5756,16 +5591,16 @@
         <v>143.5338988584734</v>
       </c>
       <c r="T26" t="n">
-        <v>-0.04792455774459092</v>
+        <v>-0.05581912705726289</v>
       </c>
       <c r="U26" t="n">
-        <v>0.1151893676665339</v>
+        <v>0.05907532106844227</v>
       </c>
       <c r="V26" t="n">
-        <v>0.450366683836871</v>
+        <v>0.5305288649189612</v>
       </c>
       <c r="W26" t="n">
-        <v>0.3283170735447052</v>
+        <v>0.3830635383788834</v>
       </c>
       <c r="X26" t="n">
         <v>0.00616</v>
@@ -5775,7 +5610,7 @@
       </c>
       <c r="AC26" t="inlineStr">
         <is>
-          <t>2026-09-04T22:51:02.817759+00:00</t>
+          <t>2026-09-05T00:27:34.215537+00:00</t>
         </is>
       </c>
       <c r="AD26" t="inlineStr">
@@ -5808,9 +5643,6 @@
       <c r="E27" t="n">
         <v>1571225468928</v>
       </c>
-      <c r="F27" t="n">
-        <v>616.77001953125</v>
-      </c>
       <c r="G27" t="n">
         <v>228246994944</v>
       </c>
@@ -5848,16 +5680,16 @@
         <v>72.89843181891389</v>
       </c>
       <c r="T27" t="n">
-        <v>0.04755676931765684</v>
+        <v>0.03867739929235592</v>
       </c>
       <c r="U27" t="n">
-        <v>0.04104828038648711</v>
+        <v>-0.02601146390986653</v>
       </c>
       <c r="V27" t="n">
-        <v>-0.06464085554432875</v>
+        <v>-0.08380733014132546</v>
       </c>
       <c r="W27" t="n">
-        <v>-0.173456945027455</v>
+        <v>-0.1687382200858099</v>
       </c>
       <c r="X27" t="n">
         <v>0.00148</v>
@@ -5867,7 +5699,7 @@
       </c>
       <c r="AC27" t="inlineStr">
         <is>
-          <t>2026-09-04T22:50:57.862583+00:00</t>
+          <t>2026-09-05T00:27:30.714847+00:00</t>
         </is>
       </c>
       <c r="AD27" t="inlineStr">
@@ -5900,9 +5732,6 @@
       <c r="E28" t="n">
         <v>269231767552</v>
       </c>
-      <c r="F28" t="n">
-        <v>252.0899963378906</v>
-      </c>
       <c r="G28" t="n">
         <v>5155999744</v>
       </c>
@@ -5940,16 +5769,16 @@
         <v>201.7473016170204</v>
       </c>
       <c r="T28" t="n">
-        <v>-0.08190688081505881</v>
+        <v>-0.1353364754459454</v>
       </c>
       <c r="U28" t="n">
-        <v>-0.2648937050652613</v>
+        <v>-0.3834129858871715</v>
       </c>
       <c r="V28" t="n">
-        <v>1.089951837155252</v>
+        <v>0.9546369764311893</v>
       </c>
       <c r="W28" t="n">
-        <v>0.8607174807184335</v>
+        <v>0.8459138618007902</v>
       </c>
       <c r="X28" t="n">
         <v>0.00068999996</v>
@@ -5959,7 +5788,7 @@
       </c>
       <c r="AC28" t="inlineStr">
         <is>
-          <t>2026-09-04T22:50:59.684261+00:00</t>
+          <t>2026-09-05T00:27:31.915249+00:00</t>
         </is>
       </c>
       <c r="AD28" t="inlineStr">
@@ -5992,9 +5821,6 @@
       <c r="E29" t="n">
         <v>218200522752</v>
       </c>
-      <c r="F29" t="n">
-        <v>213.1000061035156</v>
-      </c>
       <c r="G29" t="n">
         <v>5396145152</v>
       </c>
@@ -6029,16 +5855,16 @@
         <v>109.3525666162613</v>
       </c>
       <c r="T29" t="n">
-        <v>0.01543889013504685</v>
+        <v>0.01775400046552233</v>
       </c>
       <c r="U29" t="n">
-        <v>0.2703049083535807</v>
+        <v>0.1957890844947587</v>
       </c>
       <c r="V29" t="n">
-        <v>1.000187763021298</v>
+        <v>1.109203346573487</v>
       </c>
       <c r="W29" t="n">
-        <v>1.066624744395116</v>
+        <v>1.081026087801699</v>
       </c>
       <c r="X29" t="n">
         <v>0.014520001</v>
@@ -6048,7 +5874,7 @@
       </c>
       <c r="AC29" t="inlineStr">
         <is>
-          <t>2026-09-04T22:50:55.638491+00:00</t>
+          <t>2026-09-05T00:27:29.324569+00:00</t>
         </is>
       </c>
       <c r="AD29" t="inlineStr">
@@ -6081,9 +5907,6 @@
       <c r="E30" t="n">
         <v>146043338752</v>
       </c>
-      <c r="F30" t="n">
-        <v>141.2599945068359</v>
-      </c>
       <c r="G30" t="n">
         <v>14732000256</v>
       </c>
@@ -6121,16 +5944,16 @@
         <v>28.36137190099243</v>
       </c>
       <c r="T30" t="n">
-        <v>0.2050843971658902</v>
+        <v>0.2323514228039465</v>
       </c>
       <c r="U30" t="n">
-        <v>0.2562027420227877</v>
+        <v>0.2197553250118218</v>
       </c>
       <c r="V30" t="n">
-        <v>0.1734507204669762</v>
+        <v>0.2786755274674952</v>
       </c>
       <c r="W30" t="n">
-        <v>-0.2139646206538069</v>
+        <v>-0.2082164571123949</v>
       </c>
       <c r="X30" t="n">
         <v>0.00174</v>
@@ -6140,7 +5963,7 @@
       </c>
       <c r="AC30" t="inlineStr">
         <is>
-          <t>2026-09-04T22:51:03.215115+00:00</t>
+          <t>2026-09-05T00:27:34.484110+00:00</t>
         </is>
       </c>
       <c r="AD30" t="inlineStr">
@@ -6173,9 +5996,6 @@
       <c r="E31" t="n">
         <v>457361195008</v>
       </c>
-      <c r="F31" t="n">
-        <v>158.7799987792969</v>
-      </c>
       <c r="G31" t="n">
         <v>67356999680</v>
       </c>
@@ -6210,16 +6030,16 @@
         <v>6.7901063</v>
       </c>
       <c r="T31" t="n">
-        <v>0.09966063751282261</v>
+        <v>0.05695064827864349</v>
       </c>
       <c r="U31" t="n">
-        <v>-0.2543410755947145</v>
+        <v>-0.3459596581294039</v>
       </c>
       <c r="V31" t="n">
-        <v>0.03294055845345478</v>
+        <v>0.01802043187562985</v>
       </c>
       <c r="W31" t="n">
-        <v>-0.2798667943267172</v>
+        <v>-0.3027715603406645</v>
       </c>
       <c r="X31" t="n">
         <v>0.40498</v>
@@ -6229,7 +6049,7 @@
       </c>
       <c r="AC31" t="inlineStr">
         <is>
-          <t>2026-09-04T22:50:58.309892+00:00</t>
+          <t>2026-09-05T00:27:31.031329+00:00</t>
         </is>
       </c>
       <c r="AD31" t="inlineStr">
@@ -6459,7 +6279,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TER</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -6488,7 +6308,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -6517,7 +6337,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>TER</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -6546,18 +6366,23 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>100</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="C10" t="n">
-        <v>100</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
           <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>eps_growth</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -6575,23 +6400,18 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PATH</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>94.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="C11" t="n">
-        <v>94.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
           <t>HIGH</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>eps_growth</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -6754,7 +6574,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ACMR</t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -6770,7 +6590,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>price_to_fcf</t>
+          <t>eps_growth</t>
         </is>
       </c>
       <c r="G17" t="n">
@@ -6788,18 +6608,23 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>SNOW</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>100</v>
+        <v>88.2</v>
       </c>
       <c r="C18" t="n">
-        <v>100</v>
+        <v>88.2</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
           <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>eps_growth, pe_ratio</t>
         </is>
       </c>
       <c r="G18" t="n">
@@ -6817,23 +6642,18 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>94.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="C19" t="n">
-        <v>94.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
           <t>HIGH</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>eps_growth</t>
         </is>
       </c>
       <c r="G19" t="n">
@@ -6851,7 +6671,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -6867,7 +6687,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>price_to_fcf</t>
+          <t>eps_growth</t>
         </is>
       </c>
       <c r="G20" t="n">
@@ -6885,7 +6705,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>ACMR</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -6901,7 +6721,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>eps_growth</t>
+          <t>price_to_fcf</t>
         </is>
       </c>
       <c r="G21" t="n">
@@ -6919,23 +6739,18 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SNOW</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>88.2</v>
+        <v>100</v>
       </c>
       <c r="C22" t="n">
-        <v>88.2</v>
+        <v>100</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
           <t>HIGH</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>eps_growth, pe_ratio</t>
         </is>
       </c>
       <c r="G22" t="n">
@@ -6953,7 +6768,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -6982,7 +6797,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -7011,18 +6826,23 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>100</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="C25" t="n">
-        <v>100</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
           <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>price_to_fcf</t>
         </is>
       </c>
       <c r="G25" t="n">
@@ -7299,7 +7119,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>56.02</v>
+        <v>55.21</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>

</xml_diff>